<commit_message>
Publish dashboard snapshot 2026-08-25 09:31
</commit_message>
<xml_diff>
--- a/assets/published-news.xlsx
+++ b/assets/published-news.xlsx
@@ -93,17 +93,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>www.kado.net</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C2" t="inlineStr" s="1">
         <is>
-          <t>남부지방 폭우 피해신고 2500건 넘어…사망 1명·부상 4명 추가 없어</t>
+          <t>글로벌아그로, 집중호우 등 이상기후엔 랜드콘, 메소나</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>08월18일</t>
+          <t>08월21일</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -120,17 +120,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>www.namdonews.com</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C3" t="inlineStr" s="1">
         <is>
-          <t>보성 무농약 참다래, 8월 친환경농산물 선정</t>
+          <t>종자 원, 마늘 파종기 앞두고 식용마늘의 씨마늘 둔갑 판매 우려 집중 단...</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>08월18일</t>
+          <t>08월21일</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -147,22 +147,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>www.m-i.kr</t>
+          <t>www.agrinet.co.kr</t>
         </is>
       </c>
       <c r="C4" t="inlineStr" s="1">
         <is>
-          <t>해남·진도 배추밭 400㏊ 줄인다… 작목 전환에 18억원 지원</t>
+          <t>국제종자박람회, 가수 김태연 홍보대사 위촉</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>08월18일</t>
+          <t>08월21일</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t/>
+          <t>한국농업기술진흥원</t>
         </is>
       </c>
     </row>
@@ -174,17 +174,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>www.amnews.co.kr</t>
+          <t>www.gukjenews.com</t>
         </is>
       </c>
       <c r="C5" t="inlineStr" s="1">
         <is>
-          <t>기능성 강화한 상추 신품종 '고진미'·'노을쌈' 개발</t>
+          <t>괴산 고추 축제, 세척 건 고추 1근(600g) 1만6000원 확정</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>08월18일</t>
+          <t>08월21일</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -201,17 +201,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>www.inews365.com</t>
+          <t>www.pressian.com</t>
         </is>
       </c>
       <c r="C6" t="inlineStr" s="1">
         <is>
-          <t>배추 키우고 AI로 판다…옥천 농업인 교육 10개 과정 운영</t>
+          <t>영양군, 영양 고추 H.O.T Festival 27일 개막…막바지 준비 한창</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>08월17일</t>
+          <t>08월21일</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -228,22 +228,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>www.kbsm.net</t>
+          <t>www.chukkyung.co.kr</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="1">
         <is>
-          <t>예천군, ‘젤리킹’ 여왕벌 325마리 보급…물량 1년 새 3.6배 늘어</t>
+          <t>국제종자박람회 10월 21일 개막</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>08월17일</t>
+          <t>08월21일</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t/>
+          <t>한국농업기술진흥원</t>
         </is>
       </c>
     </row>
@@ -255,17 +255,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>www.seongjuro.co.kr</t>
+          <t>www.livesnews.com</t>
         </is>
       </c>
       <c r="C8" t="inlineStr" s="1">
         <is>
-          <t>2026 하반기 종자 ·묘 유통조사 실시</t>
+          <t>NH농우바이오, 9월 추천품종 신세계꿀 참외·시너지꿀 참외·산타꿀 수박 ...</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>08월14일</t>
+          <t>08월21일</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -282,17 +282,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>www.hani.co.kr</t>
         </is>
       </c>
       <c r="C9" t="inlineStr" s="1">
         <is>
-          <t>품종보호, 지속가능한 종자산업 뒷받침…아시아·태평양 지역 권리보호...</t>
+          <t>‘고기맛 상추 ’ 나올까…엽록체가 동물성 단백질 만들었다</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>08월14일</t>
+          <t>08월21일</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -309,17 +309,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>www.ajunews.com</t>
+          <t>www.newsfreezone.co.kr</t>
         </is>
       </c>
       <c r="C10" t="inlineStr" s="1">
         <is>
-          <t>폭염·고수온에 수산 물 수급 안정 총력</t>
+          <t>배양육부터 유전자교정까지···바이오, 제약 넘어 '먹거리 산업'으로</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>08월13일</t>
+          <t>08월21일</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -336,17 +336,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>www.imaeil.com</t>
+          <t>www.nongup.net</t>
         </is>
       </c>
       <c r="C11" t="inlineStr" s="1">
         <is>
-          <t>폭염·고수온에 밥상물가 비상…정부, 농축수산 물 수급 총력 대응</t>
+          <t>양파 모종, 씨 뿌리는 시기·초기 싹 틔우기가 생육 좌우</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>08월13일</t>
+          <t>08월21일</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -363,17 +363,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>kjmbc.co.kr</t>
+          <t>www.donga.com</t>
         </is>
       </c>
       <c r="C12" t="inlineStr" s="1">
         <is>
-          <t>장성호 저수율 27%... 말라가는 농작물에 농민들 마음도 '쩍쩍'</t>
+          <t>충북, 1인가구 맞춤 ‘썬스타 수박’ 개발</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>08월13일</t>
+          <t>08월21일</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -390,17 +390,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>www.newsmaker.or.kr</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C13" t="inlineStr" s="1">
         <is>
-          <t>영광군, 콩 개화기 병해충 증가 우려…노린재·나방류 예찰 강화 당부</t>
+          <t>무 ·배추 농사, 밑거름 하나로 수확 후 저장성까지</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>08월13일</t>
+          <t>08월20일</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -417,17 +417,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>www.youngnong.co.kr</t>
+          <t>www.livesnews.com</t>
         </is>
       </c>
       <c r="C14" t="inlineStr" s="1">
         <is>
-          <t>아시아 종묘 , 청송 고추 농가 80여명에 품종 경쟁력 소개</t>
+          <t>수입 산 의존 줄이는 고랭지 토마토…‘TS판타지’ 국산 품종 주목</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>08월12일</t>
+          <t>08월20일</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -444,22 +444,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>www.betanews.net</t>
+          <t>www.youngnong.co.kr</t>
         </is>
       </c>
       <c r="C15" t="inlineStr" s="1">
         <is>
-          <t>전남광주 저탄소 농산물 인증면적 7810㏊…전국 36%</t>
+          <t>월동무 ·배추, 밑거름이 저장성 좌우…조비, 월동 작형 맞춤 비료 3종 제...</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>08월12일</t>
+          <t>08월20일</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>한국농업기술진흥원</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -471,17 +471,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>www.asiatoday.co.kr</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C16" t="inlineStr" s="1">
         <is>
-          <t>토종 '풀·꽃·나무'를 우리곁에… 전국 확산 팔걷은 농식품부</t>
+          <t>집중호우 뒤 과수 탄저병 주의… 병든 열매 따내고 즉시 방제 당부</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>08월12일</t>
+          <t>08월19일</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -498,17 +498,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>www.wonyesanup.co.kr</t>
+          <t>www.livesnews.com</t>
         </is>
       </c>
       <c r="C17" t="inlineStr" s="1">
         <is>
-          <t>농사포인트 - 기온 31℃ 이상일 때, 과실에 직사광선 노출 예상될 때 미...</t>
+          <t>종자 원, ‘식용 마늘 둔갑’ 씨마늘 유통 집중 단속</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>08월12일</t>
+          <t>08월19일</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -525,17 +525,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>www.wonyesanup.co.kr</t>
+          <t>www.hidomin.com</t>
         </is>
       </c>
       <c r="C18" t="inlineStr" s="1">
         <is>
-          <t>신기술 &amp; 새상품</t>
+          <t>국제옥수수재단, 몽골 최초 조생 다수확 하이브리드 옥수수 개발</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>08월12일</t>
+          <t>08월19일</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -552,17 +552,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>www.news1.kr</t>
+          <t>www.donga.com</t>
         </is>
       </c>
       <c r="C19" t="inlineStr" s="1">
         <is>
-          <t>폭염 견딘 안반데기 배추밭…농촌진흥청장 직접 찾아 점검</t>
+          <t>“사람 눈보다 정확” AI로 농산물 선별 ‘스마트 유통센터’ 확산</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>08월12일</t>
+          <t>08월19일</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -579,155 +579,20 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>www.mhns.co.kr</t>
+          <t>www.kado.net</t>
         </is>
       </c>
       <c r="C20" t="inlineStr" s="1">
         <is>
-          <t>경북도, 폭염으로 인한 고추 응애 발생 주의</t>
+          <t>"파프리카 5㎏이 단돈 500원" 상자째 내던져진 농심</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>08월12일</t>
+          <t>08월19일</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>www.abcn.kr</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr" s="1">
-        <is>
-          <t>폭염 시대, 30년 뒤에도 여름에 수박을 먹을 수 있을까?</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>08월12일</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>21</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>www.nongmin.com</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr" s="1">
-        <is>
-          <t>마라탕 유행에 ‘녹두’ 인기…기계수확 품종 ‘채흔’ 주목</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>08월12일</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>한국농업기술진흥원</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>22</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>www.getnews.co.kr</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr" s="1">
-        <is>
-          <t>폭염에 시금치가 '시金치'로... 8월 채소류 가격 급등에 '히트플레이션...</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>08월11일</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>23</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>sjbnews.com</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr" s="1">
-        <is>
-          <t>고창군, 농작물재해보험 ‘가을배추’ 신규 가입</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>08월10일</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>24</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>www.nongmin.com</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr" s="1">
-        <is>
-          <t>“밖은 42℃, 안은 29℃"…가락시장, 농산물 신선도 유지 ‘안간힘’</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>08월10일</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -754,11 +619,6 @@
     <hyperlink ref="C18" r:id="rId17"/>
     <hyperlink ref="C19" r:id="rId18"/>
     <hyperlink ref="C20" r:id="rId19"/>
-    <hyperlink ref="C21" r:id="rId20"/>
-    <hyperlink ref="C22" r:id="rId21"/>
-    <hyperlink ref="C23" r:id="rId22"/>
-    <hyperlink ref="C24" r:id="rId23"/>
-    <hyperlink ref="C25" r:id="rId24"/>
   </hyperlinks>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Publish dashboard snapshot 2026-08-31 09:22
</commit_message>
<xml_diff>
--- a/assets/published-news.xlsx
+++ b/assets/published-news.xlsx
@@ -93,17 +93,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>biz.heraldcorp.com</t>
         </is>
       </c>
       <c r="C2" t="inlineStr" s="1">
         <is>
-          <t>글로벌아그로, 집중호우 등 이상기후엔 랜드콘, 메소나</t>
+          <t>2026 영양 고추 H.O.T Festival ‘성료’…15만명 발길·60억 판매</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>08월21일</t>
+          <t>08월31일</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -120,17 +120,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C3" t="inlineStr" s="1">
         <is>
-          <t>종자 원, 마늘 파종기 앞두고 식용마늘의 씨마늘 둔갑 판매 우려 집중 단...</t>
+          <t>“토마토뿔나방” 포획기 종류‧설치 방법 따라 포획 효과 달라</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>08월21일</t>
+          <t>08월31일</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -147,22 +147,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>www.agrinet.co.kr</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C4" t="inlineStr" s="1">
         <is>
-          <t>국제종자박람회, 가수 김태연 홍보대사 위촉</t>
+          <t>폭염에도 대파 수확 '한창'</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>08월21일</t>
+          <t>08월31일</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>한국농업기술진흥원</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -174,17 +174,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>www.gukjenews.com</t>
+          <t>www.chosun.com</t>
         </is>
       </c>
       <c r="C5" t="inlineStr" s="1">
         <is>
-          <t>괴산 고추 축제, 세척 건 고추 1근(600g) 1만6000원 확정</t>
+          <t>추석 앞두고 농수산물 값 급등… 배추 석달새 53% 올라</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>08월21일</t>
+          <t>08월31일</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -201,22 +201,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>www.pressian.com</t>
+          <t>www.jbnews.com</t>
         </is>
       </c>
       <c r="C6" t="inlineStr" s="1">
         <is>
-          <t>영양군, 영양 고추 H.O.T Festival 27일 개막…막바지 준비 한창</t>
+          <t>남서울대 '온실 냉방 패키지 기술 ' 현장실증 성과</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>08월21일</t>
+          <t>08월30일</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t/>
+          <t>한국농업기술진흥원</t>
         </is>
       </c>
     </row>
@@ -228,22 +228,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>www.chukkyung.co.kr</t>
+          <t>www.ikpnews.net</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="1">
         <is>
-          <t>국제종자박람회 10월 21일 개막</t>
+          <t>"종자 문제" VS "잘못 키워서" 양파 흉작에 첨예한 대립</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>08월21일</t>
+          <t>08월30일</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>한국농업기술진흥원</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -255,17 +255,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>www.livesnews.com</t>
+          <t>www.sisunnews.co.kr</t>
         </is>
       </c>
       <c r="C8" t="inlineStr" s="1">
         <is>
-          <t>NH농우바이오, 9월 추천품종 신세계꿀 참외·시너지꿀 참외·산타꿀 수박 ...</t>
+          <t>2026년 08월 마지막(09월 첫째) 주 생태계 관련 정책 CHECK! [정책브리핑...</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>08월21일</t>
+          <t>08월30일</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -282,22 +282,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>www.hani.co.kr</t>
+          <t>www.wikitree.co.kr</t>
         </is>
       </c>
       <c r="C9" t="inlineStr" s="1">
         <is>
-          <t>‘고기맛 상추 ’ 나올까…엽록체가 동물성 단백질 만들었다</t>
+          <t>갈색만 있는 줄 알았는데...녹색인데 더 달고 아삭하다는 대반전 '국민...</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>08월21일</t>
+          <t>08월30일</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t/>
+          <t>(주)다농</t>
         </is>
       </c>
     </row>
@@ -309,17 +309,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>www.newsfreezone.co.kr</t>
+          <t>www.koreadaily.com</t>
         </is>
       </c>
       <c r="C10" t="inlineStr" s="1">
         <is>
-          <t>배양육부터 유전자교정까지···바이오, 제약 넘어 '먹거리 산업'으로</t>
+          <t>리콜 양상추 관련 기생충 감염 20개주로 확산</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>08월21일</t>
+          <t>08월30일</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -336,17 +336,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>www.nongup.net</t>
+          <t>www.ytn.co.kr</t>
         </is>
       </c>
       <c r="C11" t="inlineStr" s="1">
         <is>
-          <t>양파 모종, 씨 뿌리는 시기·초기 싹 틔우기가 생육 좌우</t>
+          <t>[녹색] 고온·병해충 견디는 '고랭지 배추' 품종 개발 박차</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>08월21일</t>
+          <t>08월29일</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -363,17 +363,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>www.donga.com</t>
+          <t>www.agrinet.co.kr</t>
         </is>
       </c>
       <c r="C12" t="inlineStr" s="1">
         <is>
-          <t>충북, 1인가구 맞춤 ‘썬스타 수박’ 개발</t>
+          <t>저장봄배추 여름 출하 고착화···'설 자리 잃은' 고랭지배추</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>08월21일</t>
+          <t>08월28일</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -390,17 +390,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.amnews.co.kr</t>
         </is>
       </c>
       <c r="C13" t="inlineStr" s="1">
         <is>
-          <t>무 ·배추 농사, 밑거름 하나로 수확 후 저장성까지</t>
+          <t>국립종자원, '품종보호제도‧재배심사기술' 전수</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>08월20일</t>
+          <t>08월27일</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -417,17 +417,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>www.livesnews.com</t>
+          <t>news.sbs.co.kr</t>
         </is>
       </c>
       <c r="C14" t="inlineStr" s="1">
         <is>
-          <t>수입 산 의존 줄이는 고랭지 토마토…‘TS판타지’ 국산 품종 주목</t>
+          <t>중국산 수입 김치로 조사 확대…'자연 생성' 구분 어떻게</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>08월20일</t>
+          <t>08월27일</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -444,22 +444,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>www.youngnong.co.kr</t>
+          <t>www.amnews.co.kr</t>
         </is>
       </c>
       <c r="C15" t="inlineStr" s="1">
         <is>
-          <t>월동무 ·배추, 밑거름이 저장성 좌우…조비, 월동 작형 맞춤 비료 3종 제...</t>
+          <t>잦은 비·폭염에 고개 드는 과수·원예 '탄저병'</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>08월20일</t>
+          <t>08월26일</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t/>
+          <t>(주)경농</t>
         </is>
       </c>
     </row>
@@ -471,17 +471,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.wonyesanup.co.kr</t>
         </is>
       </c>
       <c r="C16" t="inlineStr" s="1">
         <is>
-          <t>집중호우 뒤 과수 탄저병 주의… 병든 열매 따내고 즉시 방제 당부</t>
+          <t>종자원, 중남미 5개국에 '품종보호제도·재배심사기술' 전수</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>08월19일</t>
+          <t>08월26일</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -498,17 +498,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>www.livesnews.com</t>
+          <t>www.wonyesanup.co.kr</t>
         </is>
       </c>
       <c r="C17" t="inlineStr" s="1">
         <is>
-          <t>종자 원, ‘식용 마늘 둔갑’ 씨마늘 유통 집중 단속</t>
+          <t>8월 채소류 농업관측</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>08월19일</t>
+          <t>08월26일</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -525,17 +525,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>www.hidomin.com</t>
+          <t>www.wonyesanup.co.kr</t>
         </is>
       </c>
       <c r="C18" t="inlineStr" s="1">
         <is>
-          <t>국제옥수수재단, 몽골 최초 조생 다수확 하이브리드 옥수수 개발</t>
+          <t>신기술 &amp; 새상품</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>08월19일</t>
+          <t>08월26일</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -552,17 +552,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>www.donga.com</t>
+          <t>www.newspim.com</t>
         </is>
       </c>
       <c r="C19" t="inlineStr" s="1">
         <is>
-          <t>“사람 눈보다 정확” AI로 농산물 선별 ‘스마트 유통센터’ 확산</t>
+          <t>종자원, 중남미 5개국에 품종보호 기술 전수</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>08월19일</t>
+          <t>08월25일</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -579,20 +579,290 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
+          <t>www.hani.co.kr</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr" s="1">
+        <is>
+          <t>‘고기맛 상추 ’ 나올까…엽록체가 동물성 단백질 만들었다</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>08월21일</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>www.newsfreezone.co.kr</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr" s="1">
+        <is>
+          <t>배양육부터 유전자교정까지···바이오, 제약 넘어 '먹거리 산업'으로</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>08월21일</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>www.nongup.net</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr" s="1">
+        <is>
+          <t>양파 모종, 씨 뿌리는 시기·초기 싹 틔우기가 생육 좌우</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>08월21일</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>www.donga.com</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr" s="1">
+        <is>
+          <t>충북, 1인가구 맞춤 ‘썬스타 수박’ 개발</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>08월21일</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>www.newsam.co.kr</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr" s="1">
+        <is>
+          <t>무 ·배추 농사, 밑거름 하나로 수확 후 저장성까지</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>08월20일</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>www.livesnews.com</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr" s="1">
+        <is>
+          <t>수입 산 의존 줄이는 고랭지 토마토…‘TS판타지’ 국산 품종 주목</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>08월20일</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>www.youngnong.co.kr</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr" s="1">
+        <is>
+          <t>월동무 ·배추, 밑거름이 저장성 좌우…조비, 월동 작형 맞춤 비료 3종 제...</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>08월20일</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>www.newsam.co.kr</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr" s="1">
+        <is>
+          <t>집중호우 뒤 과수 탄저병 주의… 병든 열매 따내고 즉시 방제 당부</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>08월19일</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>www.hidomin.com</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr" s="1">
+        <is>
+          <t>국제옥수수재단, 몽골 최초 조생 다수확 하이브리드 옥수수 개발</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>08월19일</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>www.donga.com</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr" s="1">
+        <is>
+          <t>“사람 눈보다 정확” AI로 농산물 선별 ‘스마트 유통센터’ 확산</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>08월19일</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
           <t>www.kado.net</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr" s="1">
+      <c r="C30" t="inlineStr" s="1">
         <is>
           <t>"파프리카 5㎏이 단돈 500원" 상자째 내던져진 농심</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="D30" t="inlineStr">
         <is>
           <t>08월19일</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="E30" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -619,6 +889,16 @@
     <hyperlink ref="C18" r:id="rId17"/>
     <hyperlink ref="C19" r:id="rId18"/>
     <hyperlink ref="C20" r:id="rId19"/>
+    <hyperlink ref="C21" r:id="rId20"/>
+    <hyperlink ref="C22" r:id="rId21"/>
+    <hyperlink ref="C23" r:id="rId22"/>
+    <hyperlink ref="C24" r:id="rId23"/>
+    <hyperlink ref="C25" r:id="rId24"/>
+    <hyperlink ref="C26" r:id="rId25"/>
+    <hyperlink ref="C27" r:id="rId26"/>
+    <hyperlink ref="C28" r:id="rId27"/>
+    <hyperlink ref="C29" r:id="rId28"/>
+    <hyperlink ref="C30" r:id="rId29"/>
   </hyperlinks>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Publish dashboard snapshot 2026-09-17 13:59
</commit_message>
<xml_diff>
--- a/assets/published-news.xlsx
+++ b/assets/published-news.xlsx
@@ -93,17 +93,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>biz.heraldcorp.com</t>
+          <t>tjmbc.co.kr</t>
         </is>
       </c>
       <c r="C2" t="inlineStr" s="1">
         <is>
-          <t>2026 영양 고추 H.O.T Festival ‘성료’…15만명 발길·60억 판매</t>
+          <t>[리포트]"명절 대목 노리고.."⋯'원산지 둔갑' 또 줄줄이 적발</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>08월31일</t>
+          <t>09월17일</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -120,17 +120,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.newstopkorea.com</t>
         </is>
       </c>
       <c r="C3" t="inlineStr" s="1">
         <is>
-          <t>“토마토뿔나방” 포획기 종류‧설치 방법 따라 포획 효과 달라</t>
+          <t>[팩트체크] 청양고추의 고향은?</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>08월31일</t>
+          <t>09월17일</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -147,17 +147,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>weekly.chosun.com</t>
         </is>
       </c>
       <c r="C4" t="inlineStr" s="1">
         <is>
-          <t>폭염에도 대파 수확 '한창'</t>
+          <t>품종 개량은 되고 생명공학은 안 된다는 억지</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>08월31일</t>
+          <t>09월17일</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -174,17 +174,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>www.chosun.com</t>
+          <t>sjbnews.com</t>
         </is>
       </c>
       <c r="C5" t="inlineStr" s="1">
         <is>
-          <t>추석 앞두고 농수산물 값 급등… 배추 석달새 53% 올라</t>
+          <t>진안 무릉팜 유럽형 샐러드 상추 , 전국 곳곳에서 만난다</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>08월31일</t>
+          <t>09월16일</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -201,22 +201,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>www.jbnews.com</t>
+          <t>dream.kotra.or.kr</t>
         </is>
       </c>
       <c r="C6" t="inlineStr" s="1">
         <is>
-          <t>남서울대 '온실 냉방 패키지 기술 ' 현장실증 성과</t>
+          <t>13억 중국인을 먹여 살리는 천조 시설재배 농업 시장</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>08월30일</t>
+          <t>09월16일</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>한국농업기술진흥원</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -228,17 +228,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>www.ikpnews.net</t>
+          <t>www.hortitimes.com</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="1">
         <is>
-          <t>"종자 문제" VS "잘못 키워서" 양파 흉작에 첨예한 대립</t>
+          <t>우장춘 박사 서거 67주기, 추모 넘어 '한·일 원예 교류'로 잇다</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>08월30일</t>
+          <t>09월16일</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -255,17 +255,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>www.sisunnews.co.kr</t>
+          <t>www.the-today.com</t>
         </is>
       </c>
       <c r="C8" t="inlineStr" s="1">
         <is>
-          <t>2026년 08월 마지막(09월 첫째) 주 생태계 관련 정책 CHECK! [정책브리핑...</t>
+          <t>中허난 신샹, 과학기술·스마트화 기반 농업 현대화 가속도</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>08월30일</t>
+          <t>09월13일</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -282,22 +282,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>www.wikitree.co.kr</t>
+          <t>www.jemin.com</t>
         </is>
       </c>
       <c r="C9" t="inlineStr" s="1">
         <is>
-          <t>갈색만 있는 줄 알았는데...녹색인데 더 달고 아삭하다는 대반전 '국민...</t>
+          <t>인공지능 병해충 감시체계 전국 우수사례 인정</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>08월30일</t>
+          <t>09월13일</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>(주)다농</t>
+          <t>한국농업기술진흥원</t>
         </is>
       </c>
     </row>
@@ -309,17 +309,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>www.koreadaily.com</t>
+          <t>www.yonhapnewstv.co.kr</t>
         </is>
       </c>
       <c r="C10" t="inlineStr" s="1">
         <is>
-          <t>리콜 양상추 관련 기생충 감염 20개주로 확산</t>
+          <t>[프리즘] 뜨거워진 지구…'산업 지도'도 바꾼다</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>08월30일</t>
+          <t>09월13일</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -336,17 +336,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>www.ytn.co.kr</t>
+          <t>www.newspim.com</t>
         </is>
       </c>
       <c r="C11" t="inlineStr" s="1">
         <is>
-          <t>[녹색] 고온·병해충 견디는 '고랭지 배추' 품종 개발 박차</t>
+          <t>[농협의 농업혁신] ① 농민은 생산만 한다…선별부터 판매까지 책임지는...</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>08월29일</t>
+          <t>09월13일</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -363,17 +363,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>www.agrinet.co.kr</t>
+          <t>www.ohmynews.com</t>
         </is>
       </c>
       <c r="C12" t="inlineStr" s="1">
         <is>
-          <t>저장봄배추 여름 출하 고착화···'설 자리 잃은' 고랭지배추</t>
+          <t>42년 외길.... 백합으로 농가 살린 태안 '백합 박사'</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>08월28일</t>
+          <t>09월12일</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -390,17 +390,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>www.amnews.co.kr</t>
+          <t>www.khan.co.kr</t>
         </is>
       </c>
       <c r="C13" t="inlineStr" s="1">
         <is>
-          <t>국립종자원, '품종보호제도‧재배심사기술' 전수</t>
+          <t>“가을도 씨 뿌리기 좋은 계절”…가을 파종 7가지 무패 전략</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>08월27일</t>
+          <t>09월12일</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -417,17 +417,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>news.sbs.co.kr</t>
+          <t>www.agrinet.co.kr</t>
         </is>
       </c>
       <c r="C14" t="inlineStr" s="1">
         <is>
-          <t>중국산 수입 김치로 조사 확대…'자연 생성' 구분 어떻게</t>
+          <t>농산물가격안정제, 아쉬움이 큰 이유</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>08월27일</t>
+          <t>09월11일</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -444,22 +444,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>www.amnews.co.kr</t>
+          <t>www.farmnmarket.com</t>
         </is>
       </c>
       <c r="C15" t="inlineStr" s="1">
         <is>
-          <t>잦은 비·폭염에 고개 드는 과수·원예 '탄저병'</t>
+          <t>배추 반쪽시들음병 저항성 후보 65개체 찾았다</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>08월26일</t>
+          <t>09월11일</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>(주)경농</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -471,17 +471,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>www.wonyesanup.co.kr</t>
+          <t>www.the-stock.kr</t>
         </is>
       </c>
       <c r="C16" t="inlineStr" s="1">
         <is>
-          <t>종자원, 중남미 5개국에 '품종보호제도·재배심사기술' 전수</t>
+          <t>제놀루션, 수박 등 박과작물 바이러스 방제 특허 출원</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>08월26일</t>
+          <t>09월10일</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -498,17 +498,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>www.wonyesanup.co.kr</t>
+          <t>www.amnews.co.kr</t>
         </is>
       </c>
       <c r="C17" t="inlineStr" s="1">
         <is>
-          <t>8월 채소류 농업관측</t>
+          <t>동오시드, 겨울 오이 신품종 '다복향'</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>08월26일</t>
+          <t>09월10일</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -525,17 +525,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>www.wonyesanup.co.kr</t>
+          <t>www.mdtoday.co.kr</t>
         </is>
       </c>
       <c r="C18" t="inlineStr" s="1">
         <is>
-          <t>신기술 &amp; 새상품</t>
+          <t>제놀루션, 수박 바이러스 겨냥 RNAi 기술 특허…감염률 70% 낮춰</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>08월26일</t>
+          <t>09월10일</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -552,17 +552,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>www.newspim.com</t>
+          <t>www.edaily.co.kr</t>
         </is>
       </c>
       <c r="C19" t="inlineStr" s="1">
         <is>
-          <t>종자원, 중남미 5개국에 품종보호 기술 전수</t>
+          <t>이상기후에…스마트팜 4년간 '여의도 11배' 늘었다</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>08월25일</t>
+          <t>09월10일</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -579,17 +579,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>www.hani.co.kr</t>
+          <t>www.hankookilbo.com</t>
         </is>
       </c>
       <c r="C20" t="inlineStr" s="1">
         <is>
-          <t>‘고기맛 상추 ’ 나올까…엽록체가 동물성 단백질 만들었다</t>
+          <t>달콤한 과즙이 가득 '고창 멜론'</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>08월21일</t>
+          <t>09월10일</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -606,17 +606,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>www.newsfreezone.co.kr</t>
+          <t>www.kdfnews.com</t>
         </is>
       </c>
       <c r="C21" t="inlineStr" s="1">
         <is>
-          <t>배양육부터 유전자교정까지···바이오, 제약 넘어 '먹거리 산업'으로</t>
+          <t>日 가고시마 농업에 AI 로봇… 오이 수확부터 비료 공급까지 자동화 [KDF...</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>08월21일</t>
+          <t>09월10일</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -633,22 +633,22 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>www.nongup.net</t>
+          <t>news.tf.co.kr</t>
         </is>
       </c>
       <c r="C22" t="inlineStr" s="1">
         <is>
-          <t>양파 모종, 씨 뿌리는 시기·초기 싹 틔우기가 생육 좌우</t>
+          <t>대동, 산업부 주관 '무인 농작업 로봇' 연구개발 총괄 기업 선정</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>08월21일</t>
+          <t>09월09일</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t/>
+          <t>한국농업기술진흥원</t>
         </is>
       </c>
     </row>
@@ -660,17 +660,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>www.donga.com</t>
+          <t>www.wikitree.co.kr</t>
         </is>
       </c>
       <c r="C23" t="inlineStr" s="1">
         <is>
-          <t>충북, 1인가구 맞춤 ‘썬스타 수박’ 개발</t>
+          <t>통째로 팔던 시대는 끝났다… 두 달 만에 매출 184% 상승한 '이 상품'</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>08월21일</t>
+          <t>09월09일</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -687,17 +687,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.yonhapnewstv.co.kr</t>
         </is>
       </c>
       <c r="C24" t="inlineStr" s="1">
         <is>
-          <t>무 ·배추 농사, 밑거름 하나로 수확 후 저장성까지</t>
+          <t>중국에 뒤처진 일본…과일·채소 신품종 출원 18년 새 64%↓</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>08월20일</t>
+          <t>09월08일</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -714,17 +714,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>www.livesnews.com</t>
+          <t>www.dynews.co.kr</t>
         </is>
       </c>
       <c r="C25" t="inlineStr" s="1">
         <is>
-          <t>수입 산 의존 줄이는 고랭지 토마토…‘TS판타지’ 국산 품종 주목</t>
+          <t>현장에서/ 기후변화에 흔들리지 않는 수박, 품종에서 답을 찾다</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>08월20일</t>
+          <t>09월08일</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -741,17 +741,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>www.youngnong.co.kr</t>
+          <t>www.newsis.com</t>
         </is>
       </c>
       <c r="C26" t="inlineStr" s="1">
         <is>
-          <t>월동무 ·배추, 밑거름이 저장성 좌우…조비, 월동 작형 맞춤 비료 3종 제...</t>
+          <t>양파값 전망, 5월엔 오차 21.9%…AI로 '예측 사각지대' 보완</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>08월20일</t>
+          <t>09월08일</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -768,17 +768,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.khan.co.kr</t>
         </is>
       </c>
       <c r="C27" t="inlineStr" s="1">
         <is>
-          <t>집중호우 뒤 과수 탄저병 주의… 병든 열매 따내고 즉시 방제 당부</t>
+          <t>멀쩡한 무를 잘랐는데 ‘파란 속살’…곰팡이일까, 상한 걸까?</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>08월19일</t>
+          <t>09월06일</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -795,17 +795,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>www.hidomin.com</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C28" t="inlineStr" s="1">
         <is>
-          <t>국제옥수수재단, 몽골 최초 조생 다수확 하이브리드 옥수수 개발</t>
+          <t>아시아종묘, 국립 종자 원 기후변화 대응 실증시험포 사업 참여</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>08월19일</t>
+          <t>09월03일</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -822,17 +822,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>www.donga.com</t>
+          <t>www.g-enews.com</t>
         </is>
       </c>
       <c r="C29" t="inlineStr" s="1">
         <is>
-          <t>“사람 눈보다 정확” AI로 농산물 선별 ‘스마트 유통센터’ 확산</t>
+          <t>"14억 먹거리 생명줄 지킨다"… 中, 첫 '농지보호법' 제정해 경작지 축소...</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>08월19일</t>
+          <t>09월02일</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -849,20 +849,128 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>www.kado.net</t>
+          <t>www.agrinet.co.kr</t>
         </is>
       </c>
       <c r="C30" t="inlineStr" s="1">
         <is>
-          <t>"파프리카 5㎏이 단돈 500원" 상자째 내던져진 농심</t>
+          <t>기존 감귤 하우스에서 '저수고 바나나' 재배</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>08월19일</t>
+          <t>09월01일</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>www.youngnong.co.kr</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr" s="1">
+        <is>
+          <t>아시아종묘, 기후변화 대응 품종 개발 '현장 실증' 강화</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>09월01일</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>www.etnews.com</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr" s="1">
+        <is>
+          <t>익은 상추만 쏙쏙…사람 대신 수확하는 로봇</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>09월01일</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>www.nongmin.com</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr" s="1">
+        <is>
+          <t>골칫거리 해충 ‘토마토뿔나방’ 잡을 땐…“43W 전격 살충기 사용하세...</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>08월31일</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>www.aflnews.co.kr</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr" s="1">
+        <is>
+          <t>도프, 배추 생육용자재 '배추 결구대장' 출시</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>08월31일</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -899,6 +1007,10 @@
     <hyperlink ref="C28" r:id="rId27"/>
     <hyperlink ref="C29" r:id="rId28"/>
     <hyperlink ref="C30" r:id="rId29"/>
+    <hyperlink ref="C31" r:id="rId30"/>
+    <hyperlink ref="C32" r:id="rId31"/>
+    <hyperlink ref="C33" r:id="rId32"/>
+    <hyperlink ref="C34" r:id="rId33"/>
   </hyperlinks>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Publish dashboard snapshot 2026-09-18 14:03
</commit_message>
<xml_diff>
--- a/assets/published-news.xlsx
+++ b/assets/published-news.xlsx
@@ -93,17 +93,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>tjmbc.co.kr</t>
+          <t>www.youthdaily.co.kr</t>
         </is>
       </c>
       <c r="C2" t="inlineStr" s="1">
         <is>
-          <t>[리포트]"명절 대목 노리고.."⋯'원산지 둔갑' 또 줄줄이 적발</t>
+          <t>추석 차례상 비용 "40만원" 육박... 대형마트, 생산지 다변화에도 납품...</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>09월17일</t>
+          <t>09월18일</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -120,17 +120,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>www.newstopkorea.com</t>
+          <t>imnews.imbc.com</t>
         </is>
       </c>
       <c r="C3" t="inlineStr" s="1">
         <is>
-          <t>[팩트체크] 청양고추의 고향은?</t>
+          <t>태풍 또 일본으로 틀었다‥"도쿄 22일째 비"</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>09월17일</t>
+          <t>09월18일</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -147,12 +147,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>weekly.chosun.com</t>
+          <t>www.idaegu.co.kr</t>
         </is>
       </c>
       <c r="C4" t="inlineStr" s="1">
         <is>
-          <t>품종 개량은 되고 생명공학은 안 된다는 억지</t>
+          <t>영주시, 과수원 농업 용 로봇 실증 나선다</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -162,7 +162,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t/>
+          <t>한국농업기술진흥원</t>
         </is>
       </c>
     </row>
@@ -179,12 +179,12 @@
       </c>
       <c r="C5" t="inlineStr" s="1">
         <is>
-          <t>진안 무릉팜 유럽형 샐러드 상추 , 전국 곳곳에서 만난다</t>
+          <t>무주군 고랭지 채소 안정 생산 시범 사업 추진</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>09월16일</t>
+          <t>09월17일</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -201,17 +201,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>dream.kotra.or.kr</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C6" t="inlineStr" s="1">
         <is>
-          <t>13억 중국인을 먹여 살리는 천조 시설재배 농업 시장</t>
+          <t>신젠타코리아, 선충·토양병 동시 관리 '바니바Ⓡ 액상수화제' 내년 출...</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>09월16일</t>
+          <t>09월17일</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -228,17 +228,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>www.hortitimes.com</t>
+          <t>www.iusm.co.kr</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="1">
         <is>
-          <t>우장춘 박사 서거 67주기, 추모 넘어 '한·일 원예 교류'로 잇다</t>
+          <t>[기획] 꽃밭 너머 연구소와 시험장…영국 원예산업의 심장</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>09월16일</t>
+          <t>09월17일</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -255,17 +255,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>www.the-today.com</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C8" t="inlineStr" s="1">
         <is>
-          <t>中허난 신샹, 과학기술·스마트화 기반 농업 현대화 가속도</t>
+          <t>아시아종묘, 조생·고품질 양배추 신품종 2종 품종보호출원</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>09월13일</t>
+          <t>09월17일</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -282,22 +282,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>www.jemin.com</t>
+          <t>www.newstree.kr</t>
         </is>
       </c>
       <c r="C9" t="inlineStr" s="1">
         <is>
-          <t>인공지능 병해충 감시체계 전국 우수사례 인정</t>
+          <t>미세플라스틱이 농경지의 '트로이 목마'..오염물질·미생물 옮긴다</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>09월13일</t>
+          <t>09월17일</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>한국농업기술진흥원</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -309,17 +309,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>www.yonhapnewstv.co.kr</t>
+          <t>sjbnews.com</t>
         </is>
       </c>
       <c r="C10" t="inlineStr" s="1">
         <is>
-          <t>[프리즘] 뜨거워진 지구…'산업 지도'도 바꾼다</t>
+          <t>진안 무릉팜 유럽형 샐러드 상추 , 전국 곳곳에서 만난다</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>09월13일</t>
+          <t>09월16일</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -336,17 +336,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>www.newspim.com</t>
+          <t>www.hortitimes.com</t>
         </is>
       </c>
       <c r="C11" t="inlineStr" s="1">
         <is>
-          <t>[농협의 농업혁신] ① 농민은 생산만 한다…선별부터 판매까지 책임지는...</t>
+          <t>우장춘 박사 서거 67주기, 추모 넘어 '한·일 원예 교류'로 잇다</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>09월13일</t>
+          <t>09월16일</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">

</xml_diff>

<commit_message>
Publish dashboard snapshot 2026-09-21 11:50
</commit_message>
<xml_diff>
--- a/assets/published-news.xlsx
+++ b/assets/published-news.xlsx
@@ -93,12 +93,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>www.youthdaily.co.kr</t>
+          <t>www.mk.co.kr</t>
         </is>
       </c>
       <c r="C2" t="inlineStr" s="1">
         <is>
-          <t>추석 차례상 비용 "40만원" 육박... 대형마트, 생산지 다변화에도 납품...</t>
+          <t>폭염은 끝났는데 이제 기름값이 문제…휘발유·경유 부담 다시 커진다</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -120,12 +120,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>imnews.imbc.com</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C3" t="inlineStr" s="1">
         <is>
-          <t>태풍 또 일본으로 틀었다‥"도쿄 22일째 비"</t>
+          <t>농안법 개정안 시행… 마늘·양파 단체 "실질적 가격안전망 구축하라"</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -147,22 +147,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>www.idaegu.co.kr</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C4" t="inlineStr" s="1">
         <is>
-          <t>영주시, 과수원 농업 용 로봇 실증 나선다</t>
+          <t>[주목] 제값 못 받는 농산물…"문제는 폭리 아니라 유통비용 왜곡"</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>09월17일</t>
+          <t>09월18일</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>한국농업기술진흥원</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -174,17 +174,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>sjbnews.com</t>
+          <t>kr.people.com.cn</t>
         </is>
       </c>
       <c r="C5" t="inlineStr" s="1">
         <is>
-          <t>무주군 고랭지 채소 안정 생산 시범 사업 추진</t>
+          <t>中, “전국 재배업 발전 ‘제15차 5개년’ 계획” 배포</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>09월17일</t>
+          <t>09월18일</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -201,17 +201,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>www.youngnong.co.kr</t>
         </is>
       </c>
       <c r="C6" t="inlineStr" s="1">
         <is>
-          <t>신젠타코리아, 선충·토양병 동시 관리 '바니바Ⓡ 액상수화제' 내년 출...</t>
+          <t>주목받는 농산물 수확후처리기술… K-애그테크 핵심 부상</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>09월17일</t>
+          <t>09월18일</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -228,17 +228,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>www.iusm.co.kr</t>
+          <t>www.youthdaily.co.kr</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="1">
         <is>
-          <t>[기획] 꽃밭 너머 연구소와 시험장…영국 원예산업의 심장</t>
+          <t>추석 차례상 비용 "40만원" 육박... 대형마트, 생산지 다변화에도 납품...</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>09월17일</t>
+          <t>09월18일</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -255,17 +255,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>imnews.imbc.com</t>
         </is>
       </c>
       <c r="C8" t="inlineStr" s="1">
         <is>
-          <t>아시아종묘, 조생·고품질 양배추 신품종 2종 품종보호출원</t>
+          <t>태풍 또 일본으로 틀었다‥"도쿄 22일째 비"</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>09월17일</t>
+          <t>09월18일</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -282,12 +282,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>www.newstree.kr</t>
+          <t>www.idaegu.co.kr</t>
         </is>
       </c>
       <c r="C9" t="inlineStr" s="1">
         <is>
-          <t>미세플라스틱이 농경지의 '트로이 목마'..오염물질·미생물 옮긴다</t>
+          <t>영주시, 과수원 농업 용 로봇 실증 나선다</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -297,7 +297,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t/>
+          <t>한국농업기술진흥원</t>
         </is>
       </c>
     </row>
@@ -314,12 +314,12 @@
       </c>
       <c r="C10" t="inlineStr" s="1">
         <is>
-          <t>진안 무릉팜 유럽형 샐러드 상추 , 전국 곳곳에서 만난다</t>
+          <t>무주군 고랭지 채소 안정 생산 시범 사업 추진</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>09월16일</t>
+          <t>09월17일</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -336,17 +336,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>www.hortitimes.com</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C11" t="inlineStr" s="1">
         <is>
-          <t>우장춘 박사 서거 67주기, 추모 넘어 '한·일 원예 교류'로 잇다</t>
+          <t>신젠타코리아, 선충·토양병 동시 관리 '바니바Ⓡ 액상수화제' 내년 출...</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>09월16일</t>
+          <t>09월17일</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -363,17 +363,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>www.ohmynews.com</t>
+          <t>www.iusm.co.kr</t>
         </is>
       </c>
       <c r="C12" t="inlineStr" s="1">
         <is>
-          <t>42년 외길.... 백합으로 농가 살린 태안 '백합 박사'</t>
+          <t>[기획] 꽃밭 너머 연구소와 시험장…영국 원예산업의 심장</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>09월12일</t>
+          <t>09월17일</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -390,17 +390,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>www.khan.co.kr</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C13" t="inlineStr" s="1">
         <is>
-          <t>“가을도 씨 뿌리기 좋은 계절”…가을 파종 7가지 무패 전략</t>
+          <t>아시아종묘, 조생·고품질 양배추 신품종 2종 품종보호출원</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>09월12일</t>
+          <t>09월17일</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -417,17 +417,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>www.agrinet.co.kr</t>
+          <t>www.newstree.kr</t>
         </is>
       </c>
       <c r="C14" t="inlineStr" s="1">
         <is>
-          <t>농산물가격안정제, 아쉬움이 큰 이유</t>
+          <t>미세플라스틱이 농경지의 '트로이 목마'..오염물질·미생물 옮긴다</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>09월11일</t>
+          <t>09월17일</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">

</xml_diff>

<commit_message>
Publish dashboard snapshot 2026-09-29 09:58
</commit_message>
<xml_diff>
--- a/assets/published-news.xlsx
+++ b/assets/published-news.xlsx
@@ -93,17 +93,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>www.mk.co.kr</t>
+          <t>www.newsis.com</t>
         </is>
       </c>
       <c r="C2" t="inlineStr" s="1">
         <is>
-          <t>폭염은 끝났는데 이제 기름값이 문제…휘발유·경유 부담 다시 커진다</t>
+          <t>제8회 부산도시농업 어울마당, 내달 2~3일 개최</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>09월18일</t>
+          <t>09월28일</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -120,17 +120,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>www.idaegu.co.kr</t>
         </is>
       </c>
       <c r="C3" t="inlineStr" s="1">
         <is>
-          <t>농안법 개정안 시행… 마늘·양파 단체 "실질적 가격안전망 구축하라"</t>
+          <t>스마트농업 날개 단 성주 참외 , 조수입 6천529억 '역대 최고'</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>09월18일</t>
+          <t>09월27일</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -147,22 +147,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>sjbnews.com</t>
         </is>
       </c>
       <c r="C4" t="inlineStr" s="1">
         <is>
-          <t>[주목] 제값 못 받는 농산물…"문제는 폭리 아니라 유통비용 왜곡"</t>
+          <t>진안군, 지역 특화작목 멜론 홍콩 수출</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>09월18일</t>
+          <t>09월27일</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t/>
+          <t>농협종묘센터</t>
         </is>
       </c>
     </row>
@@ -174,17 +174,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>kr.people.com.cn</t>
+          <t>www.asiatoday.co.kr</t>
         </is>
       </c>
       <c r="C5" t="inlineStr" s="1">
         <is>
-          <t>中, “전국 재배업 발전 ‘제15차 5개년’ 계획” 배포</t>
+          <t>K과일·채소 뭉쳐야산다… 품질·매출 다 잡은 공동경영체의 힘</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>09월18일</t>
+          <t>09월27일</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -201,17 +201,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>www.youngnong.co.kr</t>
+          <t>www.pinpointnews.co.kr</t>
         </is>
       </c>
       <c r="C6" t="inlineStr" s="1">
         <is>
-          <t>주목받는 농산물 수확후처리기술… K-애그테크 핵심 부상</t>
+          <t>포름알데히드 배추 파문에 염색 상추 까지…중국, 식품법 전면 개정</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>09월18일</t>
+          <t>09월26일</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -228,17 +228,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>www.youthdaily.co.kr</t>
+          <t>www.khan.co.kr</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="1">
         <is>
-          <t>추석 차례상 비용 "40만원" 육박... 대형마트, 생산지 다변화에도 납품...</t>
+          <t>포도 이어 감귤까지···“나뭇가지를 지켜라” 아시아 ‘과일 종자 전...</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>09월18일</t>
+          <t>09월25일</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -255,17 +255,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>imnews.imbc.com</t>
+          <t>www.mt.co.kr</t>
         </is>
       </c>
       <c r="C8" t="inlineStr" s="1">
         <is>
-          <t>태풍 또 일본으로 틀었다‥"도쿄 22일째 비"</t>
+          <t>3.2만t 버려진 정부 비축농산물…野이성권 "정부, 상황 파악 못해"</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>09월18일</t>
+          <t>09월24일</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -282,22 +282,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>www.idaegu.co.kr</t>
+          <t>www.newsis.com</t>
         </is>
       </c>
       <c r="C9" t="inlineStr" s="1">
         <is>
-          <t>영주시, 과수원 농업 용 로봇 실증 나선다</t>
+          <t>[단독] 농촌 덮친 기후재난…농업재해 복구비 2.5배 급증</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>09월17일</t>
+          <t>09월24일</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>한국농업기술진흥원</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -309,17 +309,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>sjbnews.com</t>
+          <t>www.seoul.co.kr</t>
         </is>
       </c>
       <c r="C10" t="inlineStr" s="1">
         <is>
-          <t>무주군 고랭지 채소 안정 생산 시범 사업 추진</t>
+          <t>[단독]aT, 지난해 비축 양파 83% 쓰레기 처리, 75억원 손해봤다</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>09월17일</t>
+          <t>09월23일</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -336,17 +336,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>it.donga.com</t>
         </is>
       </c>
       <c r="C11" t="inlineStr" s="1">
         <is>
-          <t>신젠타코리아, 선충·토양병 동시 관리 '바니바Ⓡ 액상수화제' 내년 출...</t>
+          <t>애그리펑션 "AI 자율주행 로봇으로 만드는 쉬운 농업" [농업이 IT(잇)다...</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>09월17일</t>
+          <t>09월23일</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -363,17 +363,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>www.iusm.co.kr</t>
+          <t>www.wonyesanup.co.kr</t>
         </is>
       </c>
       <c r="C12" t="inlineStr" s="1">
         <is>
-          <t>[기획] 꽃밭 너머 연구소와 시험장…영국 원예산업의 심장</t>
+          <t>9월 채소류 농업관측</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>09월17일</t>
+          <t>09월23일</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -390,17 +390,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C13" t="inlineStr" s="1">
         <is>
-          <t>아시아종묘, 조생·고품질 양배추 신품종 2종 품종보호출원</t>
+          <t>도프, 배추 전용 프리미엄 제품 '배추 결구대장' 출시</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>09월17일</t>
+          <t>09월22일</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -417,17 +417,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>www.newstree.kr</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C14" t="inlineStr" s="1">
         <is>
-          <t>미세플라스틱이 농경지의 '트로이 목마'..오염물질·미생물 옮긴다</t>
+          <t>가락시장 팰릿출하품 확대에 산지 ‘신음’</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>09월17일</t>
+          <t>09월21일</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -444,17 +444,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>www.farmnmarket.com</t>
+          <t>www.amnews.co.kr</t>
         </is>
       </c>
       <c r="C15" t="inlineStr" s="1">
         <is>
-          <t>배추 반쪽시들음병 저항성 후보 65개체 찾았다</t>
+          <t>농진청, 밭농업 기계화 속도 낸다</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>09월11일</t>
+          <t>09월20일</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -471,17 +471,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>www.the-stock.kr</t>
+          <t>www.mk.co.kr</t>
         </is>
       </c>
       <c r="C16" t="inlineStr" s="1">
         <is>
-          <t>제놀루션, 수박 등 박과작물 바이러스 방제 특허 출원</t>
+          <t>폭염은 끝났는데 이제 기름값이 문제…휘발유·경유 부담 다시 커진다</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>09월10일</t>
+          <t>09월18일</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -498,17 +498,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>www.amnews.co.kr</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C17" t="inlineStr" s="1">
         <is>
-          <t>동오시드, 겨울 오이 신품종 '다복향'</t>
+          <t>농안법 개정안 시행… 마늘·양파 단체 "실질적 가격안전망 구축하라"</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>09월10일</t>
+          <t>09월18일</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -525,17 +525,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>www.mdtoday.co.kr</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C18" t="inlineStr" s="1">
         <is>
-          <t>제놀루션, 수박 바이러스 겨냥 RNAi 기술 특허…감염률 70% 낮춰</t>
+          <t>[주목] 제값 못 받는 농산물…"문제는 폭리 아니라 유통비용 왜곡"</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>09월10일</t>
+          <t>09월18일</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -552,17 +552,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>www.edaily.co.kr</t>
+          <t>kr.people.com.cn</t>
         </is>
       </c>
       <c r="C19" t="inlineStr" s="1">
         <is>
-          <t>이상기후에…스마트팜 4년간 '여의도 11배' 늘었다</t>
+          <t>中, “전국 재배업 발전 ‘제15차 5개년’ 계획” 배포</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>09월10일</t>
+          <t>09월18일</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -579,17 +579,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>www.hankookilbo.com</t>
+          <t>www.youngnong.co.kr</t>
         </is>
       </c>
       <c r="C20" t="inlineStr" s="1">
         <is>
-          <t>달콤한 과즙이 가득 '고창 멜론'</t>
+          <t>주목받는 농산물 수확후처리기술… K-애그테크 핵심 부상</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>09월10일</t>
+          <t>09월18일</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -606,17 +606,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>www.kdfnews.com</t>
+          <t>www.youthdaily.co.kr</t>
         </is>
       </c>
       <c r="C21" t="inlineStr" s="1">
         <is>
-          <t>日 가고시마 농업에 AI 로봇… 오이 수확부터 비료 공급까지 자동화 [KDF...</t>
+          <t>추석 차례상 비용 "40만원" 육박... 대형마트, 생산지 다변화에도 납품...</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>09월10일</t>
+          <t>09월18일</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -633,22 +633,22 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>news.tf.co.kr</t>
+          <t>imnews.imbc.com</t>
         </is>
       </c>
       <c r="C22" t="inlineStr" s="1">
         <is>
-          <t>대동, 산업부 주관 '무인 농작업 로봇' 연구개발 총괄 기업 선정</t>
+          <t>태풍 또 일본으로 틀었다‥"도쿄 22일째 비"</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>09월09일</t>
+          <t>09월18일</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>한국농업기술진흥원</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -660,22 +660,22 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>www.wikitree.co.kr</t>
+          <t>www.idaegu.co.kr</t>
         </is>
       </c>
       <c r="C23" t="inlineStr" s="1">
         <is>
-          <t>통째로 팔던 시대는 끝났다… 두 달 만에 매출 184% 상승한 '이 상품'</t>
+          <t>영주시, 과수원 농업 용 로봇 실증 나선다</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>09월09일</t>
+          <t>09월17일</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t/>
+          <t>한국농업기술진흥원</t>
         </is>
       </c>
     </row>
@@ -687,17 +687,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>www.yonhapnewstv.co.kr</t>
+          <t>sjbnews.com</t>
         </is>
       </c>
       <c r="C24" t="inlineStr" s="1">
         <is>
-          <t>중국에 뒤처진 일본…과일·채소 신품종 출원 18년 새 64%↓</t>
+          <t>무주군 고랭지 채소 안정 생산 시범 사업 추진</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>09월08일</t>
+          <t>09월17일</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -714,17 +714,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>www.dynews.co.kr</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C25" t="inlineStr" s="1">
         <is>
-          <t>현장에서/ 기후변화에 흔들리지 않는 수박, 품종에서 답을 찾다</t>
+          <t>신젠타코리아, 선충·토양병 동시 관리 '바니바Ⓡ 액상수화제' 내년 출...</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>09월08일</t>
+          <t>09월17일</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -741,17 +741,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>www.newsis.com</t>
+          <t>www.iusm.co.kr</t>
         </is>
       </c>
       <c r="C26" t="inlineStr" s="1">
         <is>
-          <t>양파값 전망, 5월엔 오차 21.9%…AI로 '예측 사각지대' 보완</t>
+          <t>[기획] 꽃밭 너머 연구소와 시험장…영국 원예산업의 심장</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>09월08일</t>
+          <t>09월17일</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -768,17 +768,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>www.khan.co.kr</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C27" t="inlineStr" s="1">
         <is>
-          <t>멀쩡한 무를 잘랐는데 ‘파란 속살’…곰팡이일까, 상한 걸까?</t>
+          <t>아시아종묘, 조생·고품질 양배추 신품종 2종 품종보호출원</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>09월06일</t>
+          <t>09월17일</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -795,17 +795,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>www.newstree.kr</t>
         </is>
       </c>
       <c r="C28" t="inlineStr" s="1">
         <is>
-          <t>아시아종묘, 국립 종자 원 기후변화 대응 실증시험포 사업 참여</t>
+          <t>미세플라스틱이 농경지의 '트로이 목마'..오염물질·미생물 옮긴다</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>09월03일</t>
+          <t>09월17일</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -822,17 +822,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>www.g-enews.com</t>
+          <t>www.dynews.co.kr</t>
         </is>
       </c>
       <c r="C29" t="inlineStr" s="1">
         <is>
-          <t>"14억 먹거리 생명줄 지킨다"… 中, 첫 '농지보호법' 제정해 경작지 축소...</t>
+          <t>현장에서/ 기후변화에 흔들리지 않는 수박, 품종에서 답을 찾다</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>09월02일</t>
+          <t>09월08일</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -849,17 +849,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>www.agrinet.co.kr</t>
+          <t>www.newsis.com</t>
         </is>
       </c>
       <c r="C30" t="inlineStr" s="1">
         <is>
-          <t>기존 감귤 하우스에서 '저수고 바나나' 재배</t>
+          <t>양파값 전망, 5월엔 오차 21.9%…AI로 '예측 사각지대' 보완</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>09월01일</t>
+          <t>09월08일</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -876,17 +876,17 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>www.youngnong.co.kr</t>
+          <t>www.khan.co.kr</t>
         </is>
       </c>
       <c r="C31" t="inlineStr" s="1">
         <is>
-          <t>아시아종묘, 기후변화 대응 품종 개발 '현장 실증' 강화</t>
+          <t>멀쩡한 무를 잘랐는데 ‘파란 속살’…곰팡이일까, 상한 걸까?</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>09월01일</t>
+          <t>09월06일</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -903,17 +903,17 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>www.etnews.com</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C32" t="inlineStr" s="1">
         <is>
-          <t>익은 상추만 쏙쏙…사람 대신 수확하는 로봇</t>
+          <t>아시아종묘, 국립 종자 원 기후변화 대응 실증시험포 사업 참여</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>09월01일</t>
+          <t>09월03일</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -930,17 +930,17 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.g-enews.com</t>
         </is>
       </c>
       <c r="C33" t="inlineStr" s="1">
         <is>
-          <t>골칫거리 해충 ‘토마토뿔나방’ 잡을 땐…“43W 전격 살충기 사용하세...</t>
+          <t>"14억 먹거리 생명줄 지킨다"… 中, 첫 '농지보호법' 제정해 경작지 축소...</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>08월31일</t>
+          <t>09월02일</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -957,20 +957,101 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>www.agrinet.co.kr</t>
         </is>
       </c>
       <c r="C34" t="inlineStr" s="1">
         <is>
-          <t>도프, 배추 생육용자재 '배추 결구대장' 출시</t>
+          <t>기존 감귤 하우스에서 '저수고 바나나' 재배</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
+          <t>09월01일</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>www.youngnong.co.kr</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr" s="1">
+        <is>
+          <t>아시아종묘, 기후변화 대응 품종 개발 '현장 실증' 강화</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>09월01일</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>www.etnews.com</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr" s="1">
+        <is>
+          <t>익은 상추만 쏙쏙…사람 대신 수확하는 로봇</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>09월01일</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>www.nongmin.com</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr" s="1">
+        <is>
+          <t>골칫거리 해충 ‘토마토뿔나방’ 잡을 땐…“43W 전격 살충기 사용하세...</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
           <t>08월31일</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr">
+      <c r="E37" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -1011,6 +1092,9 @@
     <hyperlink ref="C32" r:id="rId31"/>
     <hyperlink ref="C33" r:id="rId32"/>
     <hyperlink ref="C34" r:id="rId33"/>
+    <hyperlink ref="C35" r:id="rId34"/>
+    <hyperlink ref="C36" r:id="rId35"/>
+    <hyperlink ref="C37" r:id="rId36"/>
   </hyperlinks>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Publish dashboard snapshot 2026-09-30 15:28
</commit_message>
<xml_diff>
--- a/assets/published-news.xlsx
+++ b/assets/published-news.xlsx
@@ -93,17 +93,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>www.newsis.com</t>
+          <t>www.m-i.kr</t>
         </is>
       </c>
       <c r="C2" t="inlineStr" s="1">
         <is>
-          <t>제8회 부산도시농업 어울마당, 내달 2~3일 개최</t>
+          <t>해남군, 시설과채류 줄기 유인 자동화…작업시간 47% 이상 단축</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>09월28일</t>
+          <t>09월30일</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -120,22 +120,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>www.idaegu.co.kr</t>
+          <t>www.ilyoseoul.co.kr</t>
         </is>
       </c>
       <c r="C3" t="inlineStr" s="1">
         <is>
-          <t>스마트농업 날개 단 성주 참외 , 조수입 6천529억 '역대 최고'</t>
+          <t>농협, 종자사업 통합 추진…NH농우바이오 중심 글로벌 경쟁력 강화</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>09월27일</t>
+          <t>09월30일</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t/>
+          <t>농협종묘센터</t>
         </is>
       </c>
     </row>
@@ -147,22 +147,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>sjbnews.com</t>
+          <t>news.sbs.co.kr</t>
         </is>
       </c>
       <c r="C4" t="inlineStr" s="1">
         <is>
-          <t>진안군, 지역 특화작목 멜론 홍콩 수출</t>
+          <t>"벌써 김장철이네"…예년보다 빨라진 '예약 경쟁'</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>09월27일</t>
+          <t>09월30일</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>농협종묘센터</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -174,17 +174,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>www.asiatoday.co.kr</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C5" t="inlineStr" s="1">
         <is>
-          <t>K과일·채소 뭉쳐야산다… 품질·매출 다 잡은 공동경영체의 힘</t>
+          <t>“내 손안의 인공지능(AI) 농사 전문가” 농촌진흥청, ‘AI 이삭이’ 2.0...</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>09월27일</t>
+          <t>09월30일</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -201,17 +201,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>www.pinpointnews.co.kr</t>
+          <t>www.youngnong.co.kr</t>
         </is>
       </c>
       <c r="C6" t="inlineStr" s="1">
         <is>
-          <t>포름알데히드 배추 파문에 염색 상추 까지…중국, 식품법 전면 개정</t>
+          <t>NH농우바이오, 겨울 수박 ·참외 겨냥 10월 추천품종 4종 제안</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>09월26일</t>
+          <t>09월30일</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -228,17 +228,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>www.khan.co.kr</t>
+          <t>www.newsjeju.net</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="1">
         <is>
-          <t>포도 이어 감귤까지···“나뭇가지를 지켜라” 아시아 ‘과일 종자 전...</t>
+          <t>성산일출봉농협 청년부, 월동무 신품종 시험재배 실시</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>09월25일</t>
+          <t>09월30일</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -255,17 +255,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>www.mt.co.kr</t>
+          <t>www.youngnong.co.kr</t>
         </is>
       </c>
       <c r="C8" t="inlineStr" s="1">
         <is>
-          <t>3.2만t 버려진 정부 비축농산물…野이성권 "정부, 상황 파악 못해"</t>
+          <t>시설채소 바이러스병 비상…경농, 매개충 차단·바이러스 예방 '이중 방...</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>09월24일</t>
+          <t>09월29일</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -282,17 +282,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>www.newsis.com</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C9" t="inlineStr" s="1">
         <is>
-          <t>[단독] 농촌 덮친 기후재난…농업재해 복구비 2.5배 급증</t>
+          <t>한국원예학회 추계학술발표회 11월4~7일 제주서</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>09월24일</t>
+          <t>09월29일</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -309,17 +309,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>www.seoul.co.kr</t>
+          <t>www.newsfarm.co.kr</t>
         </is>
       </c>
       <c r="C10" t="inlineStr" s="1">
         <is>
-          <t>[단독]aT, 지난해 비축 양파 83% 쓰레기 처리, 75억원 손해봤다</t>
+          <t>팜한농, 가을철 안정 영농 위한 '맞춤형 3종' 주목</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>09월23일</t>
+          <t>09월29일</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -336,17 +336,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>it.donga.com</t>
+          <t>www.newsfarm.co.kr</t>
         </is>
       </c>
       <c r="C11" t="inlineStr" s="1">
         <is>
-          <t>애그리펑션 "AI 자율주행 로봇으로 만드는 쉬운 농업" [농업이 IT(잇)다...</t>
+          <t>가을철 작물 위협 노균병·역병…체계적 관리 필요</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>09월23일</t>
+          <t>09월29일</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -363,17 +363,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>www.wonyesanup.co.kr</t>
+          <t>www.newsis.com</t>
         </is>
       </c>
       <c r="C12" t="inlineStr" s="1">
         <is>
-          <t>9월 채소류 농업관측</t>
+          <t>제8회 부산도시농업 어울마당, 내달 2~3일 개최</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>09월23일</t>
+          <t>09월28일</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -390,17 +390,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.idaegu.co.kr</t>
         </is>
       </c>
       <c r="C13" t="inlineStr" s="1">
         <is>
-          <t>도프, 배추 전용 프리미엄 제품 '배추 결구대장' 출시</t>
+          <t>스마트농업 날개 단 성주 참외 , 조수입 6천529억 '역대 최고'</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>09월22일</t>
+          <t>09월27일</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -417,22 +417,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>sjbnews.com</t>
         </is>
       </c>
       <c r="C14" t="inlineStr" s="1">
         <is>
-          <t>가락시장 팰릿출하품 확대에 산지 ‘신음’</t>
+          <t>진안군, 지역 특화작목 멜론 홍콩 수출</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>09월21일</t>
+          <t>09월27일</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t/>
+          <t>농협종묘센터</t>
         </is>
       </c>
     </row>
@@ -444,17 +444,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>www.amnews.co.kr</t>
+          <t>www.asiatoday.co.kr</t>
         </is>
       </c>
       <c r="C15" t="inlineStr" s="1">
         <is>
-          <t>농진청, 밭농업 기계화 속도 낸다</t>
+          <t>K과일·채소 뭉쳐야산다… 품질·매출 다 잡은 공동경영체의 힘</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>09월20일</t>
+          <t>09월27일</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -471,17 +471,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>www.mk.co.kr</t>
+          <t>www.pinpointnews.co.kr</t>
         </is>
       </c>
       <c r="C16" t="inlineStr" s="1">
         <is>
-          <t>폭염은 끝났는데 이제 기름값이 문제…휘발유·경유 부담 다시 커진다</t>
+          <t>포름알데히드 배추 파문에 염색 상추 까지…중국, 식품법 전면 개정</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>09월18일</t>
+          <t>09월26일</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -498,17 +498,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>www.khan.co.kr</t>
         </is>
       </c>
       <c r="C17" t="inlineStr" s="1">
         <is>
-          <t>농안법 개정안 시행… 마늘·양파 단체 "실질적 가격안전망 구축하라"</t>
+          <t>포도 이어 감귤까지···“나뭇가지를 지켜라” 아시아 ‘과일 종자 전...</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>09월18일</t>
+          <t>09월25일</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -525,17 +525,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>www.mt.co.kr</t>
         </is>
       </c>
       <c r="C18" t="inlineStr" s="1">
         <is>
-          <t>[주목] 제값 못 받는 농산물…"문제는 폭리 아니라 유통비용 왜곡"</t>
+          <t>3.2만t 버려진 정부 비축농산물…野이성권 "정부, 상황 파악 못해"</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>09월18일</t>
+          <t>09월24일</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -552,17 +552,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>kr.people.com.cn</t>
+          <t>www.newsis.com</t>
         </is>
       </c>
       <c r="C19" t="inlineStr" s="1">
         <is>
-          <t>中, “전국 재배업 발전 ‘제15차 5개년’ 계획” 배포</t>
+          <t>[단독] 농촌 덮친 기후재난…농업재해 복구비 2.5배 급증</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>09월18일</t>
+          <t>09월24일</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -579,17 +579,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>www.youngnong.co.kr</t>
+          <t>www.seoul.co.kr</t>
         </is>
       </c>
       <c r="C20" t="inlineStr" s="1">
         <is>
-          <t>주목받는 농산물 수확후처리기술… K-애그테크 핵심 부상</t>
+          <t>[단독]aT, 지난해 비축 양파 83% 쓰레기 처리, 75억원 손해봤다</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>09월18일</t>
+          <t>09월23일</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -606,17 +606,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>www.youthdaily.co.kr</t>
+          <t>it.donga.com</t>
         </is>
       </c>
       <c r="C21" t="inlineStr" s="1">
         <is>
-          <t>추석 차례상 비용 "40만원" 육박... 대형마트, 생산지 다변화에도 납품...</t>
+          <t>애그리펑션 "AI 자율주행 로봇으로 만드는 쉬운 농업" [농업이 IT(잇)다...</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>09월18일</t>
+          <t>09월23일</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -633,17 +633,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>imnews.imbc.com</t>
+          <t>www.wonyesanup.co.kr</t>
         </is>
       </c>
       <c r="C22" t="inlineStr" s="1">
         <is>
-          <t>태풍 또 일본으로 틀었다‥"도쿄 22일째 비"</t>
+          <t>9월 채소류 농업관측</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>09월18일</t>
+          <t>09월23일</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -660,22 +660,22 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>www.idaegu.co.kr</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C23" t="inlineStr" s="1">
         <is>
-          <t>영주시, 과수원 농업 용 로봇 실증 나선다</t>
+          <t>도프, 배추 전용 프리미엄 제품 '배추 결구대장' 출시</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>09월17일</t>
+          <t>09월22일</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>한국농업기술진흥원</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -687,17 +687,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>sjbnews.com</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C24" t="inlineStr" s="1">
         <is>
-          <t>무주군 고랭지 채소 안정 생산 시범 사업 추진</t>
+          <t>가락시장 팰릿출하품 확대에 산지 ‘신음’</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>09월17일</t>
+          <t>09월21일</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -714,17 +714,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>www.amnews.co.kr</t>
         </is>
       </c>
       <c r="C25" t="inlineStr" s="1">
         <is>
-          <t>신젠타코리아, 선충·토양병 동시 관리 '바니바Ⓡ 액상수화제' 내년 출...</t>
+          <t>농진청, 밭농업 기계화 속도 낸다</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>09월17일</t>
+          <t>09월20일</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -741,17 +741,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>www.iusm.co.kr</t>
+          <t>www.mk.co.kr</t>
         </is>
       </c>
       <c r="C26" t="inlineStr" s="1">
         <is>
-          <t>[기획] 꽃밭 너머 연구소와 시험장…영국 원예산업의 심장</t>
+          <t>폭염은 끝났는데 이제 기름값이 문제…휘발유·경유 부담 다시 커진다</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>09월17일</t>
+          <t>09월18일</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -773,12 +773,12 @@
       </c>
       <c r="C27" t="inlineStr" s="1">
         <is>
-          <t>아시아종묘, 조생·고품질 양배추 신품종 2종 품종보호출원</t>
+          <t>농안법 개정안 시행… 마늘·양파 단체 "실질적 가격안전망 구축하라"</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>09월17일</t>
+          <t>09월18일</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -795,17 +795,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>www.newstree.kr</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C28" t="inlineStr" s="1">
         <is>
-          <t>미세플라스틱이 농경지의 '트로이 목마'..오염물질·미생물 옮긴다</t>
+          <t>[주목] 제값 못 받는 농산물…"문제는 폭리 아니라 유통비용 왜곡"</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>09월17일</t>
+          <t>09월18일</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -822,17 +822,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>www.dynews.co.kr</t>
+          <t>kr.people.com.cn</t>
         </is>
       </c>
       <c r="C29" t="inlineStr" s="1">
         <is>
-          <t>현장에서/ 기후변화에 흔들리지 않는 수박, 품종에서 답을 찾다</t>
+          <t>中, “전국 재배업 발전 ‘제15차 5개년’ 계획” 배포</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>09월08일</t>
+          <t>09월18일</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -849,17 +849,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>www.newsis.com</t>
+          <t>www.youngnong.co.kr</t>
         </is>
       </c>
       <c r="C30" t="inlineStr" s="1">
         <is>
-          <t>양파값 전망, 5월엔 오차 21.9%…AI로 '예측 사각지대' 보완</t>
+          <t>주목받는 농산물 수확후처리기술… K-애그테크 핵심 부상</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>09월08일</t>
+          <t>09월18일</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -876,17 +876,17 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>www.khan.co.kr</t>
+          <t>imnews.imbc.com</t>
         </is>
       </c>
       <c r="C31" t="inlineStr" s="1">
         <is>
-          <t>멀쩡한 무를 잘랐는데 ‘파란 속살’…곰팡이일까, 상한 걸까?</t>
+          <t>태풍 또 일본으로 틀었다‥"도쿄 22일째 비"</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>09월06일</t>
+          <t>09월18일</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -903,22 +903,22 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>www.idaegu.co.kr</t>
         </is>
       </c>
       <c r="C32" t="inlineStr" s="1">
         <is>
-          <t>아시아종묘, 국립 종자 원 기후변화 대응 실증시험포 사업 참여</t>
+          <t>영주시, 과수원 농업 용 로봇 실증 나선다</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>09월03일</t>
+          <t>09월17일</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t/>
+          <t>한국농업기술진흥원</t>
         </is>
       </c>
     </row>
@@ -930,17 +930,17 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>www.g-enews.com</t>
+          <t>sjbnews.com</t>
         </is>
       </c>
       <c r="C33" t="inlineStr" s="1">
         <is>
-          <t>"14억 먹거리 생명줄 지킨다"… 中, 첫 '농지보호법' 제정해 경작지 축소...</t>
+          <t>무주군 고랭지 채소 안정 생산 시범 사업 추진</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>09월02일</t>
+          <t>09월17일</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -957,17 +957,17 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>www.agrinet.co.kr</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C34" t="inlineStr" s="1">
         <is>
-          <t>기존 감귤 하우스에서 '저수고 바나나' 재배</t>
+          <t>신젠타코리아, 선충·토양병 동시 관리 '바니바Ⓡ 액상수화제' 내년 출...</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>09월01일</t>
+          <t>09월17일</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -984,17 +984,17 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>www.youngnong.co.kr</t>
+          <t>www.iusm.co.kr</t>
         </is>
       </c>
       <c r="C35" t="inlineStr" s="1">
         <is>
-          <t>아시아종묘, 기후변화 대응 품종 개발 '현장 실증' 강화</t>
+          <t>[기획] 꽃밭 너머 연구소와 시험장…영국 원예산업의 심장</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>09월01일</t>
+          <t>09월17일</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -1011,17 +1011,17 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>www.etnews.com</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C36" t="inlineStr" s="1">
         <is>
-          <t>익은 상추만 쏙쏙…사람 대신 수확하는 로봇</t>
+          <t>아시아종묘, 조생·고품질 양배추 신품종 2종 품종보호출원</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>09월01일</t>
+          <t>09월17일</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -1038,17 +1038,17 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.newstree.kr</t>
         </is>
       </c>
       <c r="C37" t="inlineStr" s="1">
         <is>
-          <t>골칫거리 해충 ‘토마토뿔나방’ 잡을 땐…“43W 전격 살충기 사용하세...</t>
+          <t>미세플라스틱이 농경지의 '트로이 목마'..오염물질·미생물 옮긴다</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>08월31일</t>
+          <t>09월17일</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">

</xml_diff>

<commit_message>
Publish dashboard snapshot 2026-10-02 14:17
</commit_message>
<xml_diff>
--- a/assets/published-news.xlsx
+++ b/assets/published-news.xlsx
@@ -93,17 +93,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>www.m-i.kr</t>
+          <t>www.nongup.net</t>
         </is>
       </c>
       <c r="C2" t="inlineStr" s="1">
         <is>
-          <t>해남군, 시설과채류 줄기 유인 자동화…작업시간 47% 이상 단축</t>
+          <t>거베라 소비 트렌드 바뀌었다…노동 부담 줄인 신품종 공개</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>09월30일</t>
+          <t>10월02일</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -120,22 +120,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>www.ilyoseoul.co.kr</t>
+          <t>news.bizwatch.co.kr</t>
         </is>
       </c>
       <c r="C3" t="inlineStr" s="1">
         <is>
-          <t>농협, 종자사업 통합 추진…NH농우바이오 중심 글로벌 경쟁력 강화</t>
+          <t>네이버·컬리 '동맹 1년', 모두 웃었다 …다음 승부처는</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>09월30일</t>
+          <t>10월02일</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>농협종묘센터</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -147,17 +147,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>news.sbs.co.kr</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C4" t="inlineStr" s="1">
         <is>
-          <t>"벌써 김장철이네"…예년보다 빨라진 '예약 경쟁'</t>
+          <t>병해충 진단부터 영농기술 상담까지…‘AI 이삭이’ 2.0 출시</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>09월30일</t>
+          <t>10월02일</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -174,17 +174,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C5" t="inlineStr" s="1">
         <is>
-          <t>“내 손안의 인공지능(AI) 농사 전문가” 농촌진흥청, ‘AI 이삭이’ 2.0...</t>
+          <t>가을에도 밭 갈아엎는다…‘양배추’ 농가에 무슨 일이?</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>09월30일</t>
+          <t>10월02일</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -201,17 +201,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>www.youngnong.co.kr</t>
+          <t>www.segye.com</t>
         </is>
       </c>
       <c r="C6" t="inlineStr" s="1">
         <is>
-          <t>NH농우바이오, 겨울 수박 ·참외 겨냥 10월 추천품종 4종 제안</t>
+          <t>“종자 가치, 농업 시작 넘어 식량안보의 미래 결정”</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>09월30일</t>
+          <t>10월01일</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -228,17 +228,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>www.newsjeju.net</t>
+          <t>www.obsnews.co.kr</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="1">
         <is>
-          <t>성산일출봉농협 청년부, 월동무 신품종 시험재배 실시</t>
+          <t>도쿄 35일 연속 비 최장 기록…'기상병' 호소 증가</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>09월30일</t>
+          <t>10월01일</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -255,17 +255,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>www.youngnong.co.kr</t>
+          <t>www.vegannews.co.kr</t>
         </is>
       </c>
       <c r="C8" t="inlineStr" s="1">
         <is>
-          <t>시설채소 바이러스병 비상…경농, 매개충 차단·바이러스 예방 '이중 방...</t>
+          <t>씨앗 봉투 발아율은 재배 성공률과 다르다</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>09월29일</t>
+          <t>10월01일</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -282,17 +282,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.ccdn.co.kr</t>
         </is>
       </c>
       <c r="C9" t="inlineStr" s="1">
         <is>
-          <t>한국원예학회 추계학술발표회 11월4~7일 제주서</t>
+          <t>충북농기원, 중소형 수박 신품종 보급 확대</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>09월29일</t>
+          <t>10월01일</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -309,17 +309,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>www.newsfarm.co.kr</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C10" t="inlineStr" s="1">
         <is>
-          <t>팜한농, 가을철 안정 영농 위한 '맞춤형 3종' 주목</t>
+          <t>본격적인 시설재배 시작, 바이러스병 예방해야</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>09월29일</t>
+          <t>10월01일</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -336,17 +336,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>www.newsfarm.co.kr</t>
+          <t>www.kyongbuk.co.kr</t>
         </is>
       </c>
       <c r="C11" t="inlineStr" s="1">
         <is>
-          <t>가을철 작물 위협 노균병·역병…체계적 관리 필요</t>
+          <t>성주 외국인 계절근로자 연말까지 970여 명 투입…농번기 인력난 지원</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>09월29일</t>
+          <t>10월01일</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -363,17 +363,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>www.newsis.com</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C12" t="inlineStr" s="1">
         <is>
-          <t>제8회 부산도시농업 어울마당, 내달 2~3일 개최</t>
+          <t>영세성 갇힌 국내 종자 산업…"데이터 기반 신육종 지원 시급"</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>09월28일</t>
+          <t>10월01일</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -390,17 +390,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>www.idaegu.co.kr</t>
+          <t>www.farmnmarket.com</t>
         </is>
       </c>
       <c r="C13" t="inlineStr" s="1">
         <is>
-          <t>스마트농업 날개 단 성주 참외 , 조수입 6천529억 '역대 최고'</t>
+          <t>정읍시, 가을 배추· 무 병해충 초기 방제 당부</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>09월27일</t>
+          <t>10월01일</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -417,22 +417,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>sjbnews.com</t>
+          <t>www.gasnews.com</t>
         </is>
       </c>
       <c r="C14" t="inlineStr" s="1">
         <is>
-          <t>진안군, 지역 특화작목 멜론 홍콩 수출</t>
+          <t>일본LP가스협회, 시설원예 난방연료로 LP가스 채택 확산</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>09월27일</t>
+          <t>10월01일</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>농협종묘센터</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -444,17 +444,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>www.asiatoday.co.kr</t>
+          <t>www.kwnews.co.kr</t>
         </is>
       </c>
       <c r="C15" t="inlineStr" s="1">
         <is>
-          <t>K과일·채소 뭉쳐야산다… 품질·매출 다 잡은 공동경영체의 힘</t>
+          <t>계절마다 농가 덮치는 이상기후⋯강원 농업 현장 ‘비상’</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>09월27일</t>
+          <t>10월01일</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -471,17 +471,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>www.pinpointnews.co.kr</t>
+          <t>www.gnnews.co.kr</t>
         </is>
       </c>
       <c r="C16" t="inlineStr" s="1">
         <is>
-          <t>포름알데히드 배추 파문에 염색 상추 까지…중국, 식품법 전면 개정</t>
+          <t>폭염에 빈 시설, 작은 수박 이 대안 될까</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>09월26일</t>
+          <t>09월30일</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -498,17 +498,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>www.khan.co.kr</t>
+          <t>www.knnews.co.kr</t>
         </is>
       </c>
       <c r="C17" t="inlineStr" s="1">
         <is>
-          <t>포도 이어 감귤까지···“나뭇가지를 지켜라” 아시아 ‘과일 종자 전...</t>
+          <t>경남농기원, 고온기 소과종 수박 수경재배 연구</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>09월25일</t>
+          <t>09월30일</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -525,17 +525,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>www.mt.co.kr</t>
+          <t>www.sisaweek.com</t>
         </is>
       </c>
       <c r="C18" t="inlineStr" s="1">
         <is>
-          <t>3.2만t 버려진 정부 비축농산물…野이성권 "정부, 상황 파악 못해"</t>
+          <t>기후변화에 맞서는 '유전공학'… '식량난' 해법될까</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>09월24일</t>
+          <t>09월30일</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -552,22 +552,22 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>www.newsis.com</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C19" t="inlineStr" s="1">
         <is>
-          <t>[단독] 농촌 덮친 기후재난…농업재해 복구비 2.5배 급증</t>
+          <t>바이러스, 매개충 차단과 불활성화로 이중 방어막 구축</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>09월24일</t>
+          <t>09월30일</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t/>
+          <t>(주)경농</t>
         </is>
       </c>
     </row>
@@ -579,17 +579,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>www.seoul.co.kr</t>
+          <t>www.m-i.kr</t>
         </is>
       </c>
       <c r="C20" t="inlineStr" s="1">
         <is>
-          <t>[단독]aT, 지난해 비축 양파 83% 쓰레기 처리, 75억원 손해봤다</t>
+          <t>해남군, 시설과채류 줄기 유인 자동화…작업시간 47% 이상 단축</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>09월23일</t>
+          <t>09월30일</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -606,22 +606,22 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>it.donga.com</t>
+          <t>www.ilyoseoul.co.kr</t>
         </is>
       </c>
       <c r="C21" t="inlineStr" s="1">
         <is>
-          <t>애그리펑션 "AI 자율주행 로봇으로 만드는 쉬운 농업" [농업이 IT(잇)다...</t>
+          <t>농협, 종자사업 통합 추진…NH농우바이오 중심 글로벌 경쟁력 강화</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>09월23일</t>
+          <t>09월30일</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t/>
+          <t>농협종묘센터</t>
         </is>
       </c>
     </row>
@@ -633,17 +633,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>www.wonyesanup.co.kr</t>
+          <t>news.sbs.co.kr</t>
         </is>
       </c>
       <c r="C22" t="inlineStr" s="1">
         <is>
-          <t>9월 채소류 농업관측</t>
+          <t>"벌써 김장철이네"…예년보다 빨라진 '예약 경쟁'</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>09월23일</t>
+          <t>09월30일</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -665,12 +665,12 @@
       </c>
       <c r="C23" t="inlineStr" s="1">
         <is>
-          <t>도프, 배추 전용 프리미엄 제품 '배추 결구대장' 출시</t>
+          <t>“내 손안의 인공지능(AI) 농사 전문가” 농촌진흥청, ‘AI 이삭이’ 2.0...</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>09월22일</t>
+          <t>09월30일</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -687,17 +687,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.youngnong.co.kr</t>
         </is>
       </c>
       <c r="C24" t="inlineStr" s="1">
         <is>
-          <t>가락시장 팰릿출하품 확대에 산지 ‘신음’</t>
+          <t>NH농우바이오, 겨울 수박 ·참외 겨냥 10월 추천품종 4종 제안</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>09월21일</t>
+          <t>09월30일</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -714,17 +714,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>www.amnews.co.kr</t>
+          <t>www.newsjeju.net</t>
         </is>
       </c>
       <c r="C25" t="inlineStr" s="1">
         <is>
-          <t>농진청, 밭농업 기계화 속도 낸다</t>
+          <t>성산일출봉농협 청년부, 월동무 신품종 시험재배 실시</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>09월20일</t>
+          <t>09월30일</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -741,17 +741,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>www.mk.co.kr</t>
+          <t>www.youngnong.co.kr</t>
         </is>
       </c>
       <c r="C26" t="inlineStr" s="1">
         <is>
-          <t>폭염은 끝났는데 이제 기름값이 문제…휘발유·경유 부담 다시 커진다</t>
+          <t>시설채소 바이러스병 비상…경농, 매개충 차단·바이러스 예방 '이중 방...</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>09월18일</t>
+          <t>09월29일</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -768,17 +768,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C27" t="inlineStr" s="1">
         <is>
-          <t>농안법 개정안 시행… 마늘·양파 단체 "실질적 가격안전망 구축하라"</t>
+          <t>한국원예학회 추계학술발표회 11월4~7일 제주서</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>09월18일</t>
+          <t>09월29일</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -795,17 +795,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>www.newsfarm.co.kr</t>
         </is>
       </c>
       <c r="C28" t="inlineStr" s="1">
         <is>
-          <t>[주목] 제값 못 받는 농산물…"문제는 폭리 아니라 유통비용 왜곡"</t>
+          <t>팜한농, 가을철 안정 영농 위한 '맞춤형 3종' 주목</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>09월18일</t>
+          <t>09월29일</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -822,236 +822,20 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>kr.people.com.cn</t>
+          <t>www.newsfarm.co.kr</t>
         </is>
       </c>
       <c r="C29" t="inlineStr" s="1">
         <is>
-          <t>中, “전국 재배업 발전 ‘제15차 5개년’ 계획” 배포</t>
+          <t>가을철 작물 위협 노균병·역병…체계적 관리 필요</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>09월18일</t>
+          <t>09월29일</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>29</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>www.youngnong.co.kr</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr" s="1">
-        <is>
-          <t>주목받는 농산물 수확후처리기술… K-애그테크 핵심 부상</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>09월18일</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>imnews.imbc.com</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr" s="1">
-        <is>
-          <t>태풍 또 일본으로 틀었다‥"도쿄 22일째 비"</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>09월18일</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>31</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>www.idaegu.co.kr</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr" s="1">
-        <is>
-          <t>영주시, 과수원 농업 용 로봇 실증 나선다</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>09월17일</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>한국농업기술진흥원</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>32</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>sjbnews.com</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr" s="1">
-        <is>
-          <t>무주군 고랭지 채소 안정 생산 시범 사업 추진</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>09월17일</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>33</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>www.aflnews.co.kr</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr" s="1">
-        <is>
-          <t>신젠타코리아, 선충·토양병 동시 관리 '바니바Ⓡ 액상수화제' 내년 출...</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>09월17일</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>34</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>www.iusm.co.kr</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr" s="1">
-        <is>
-          <t>[기획] 꽃밭 너머 연구소와 시험장…영국 원예산업의 심장</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>09월17일</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>35</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>www.aflnews.co.kr</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr" s="1">
-        <is>
-          <t>아시아종묘, 조생·고품질 양배추 신품종 2종 품종보호출원</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>09월17일</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>36</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>www.newstree.kr</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr" s="1">
-        <is>
-          <t>미세플라스틱이 농경지의 '트로이 목마'..오염물질·미생물 옮긴다</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>09월17일</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -1087,14 +871,6 @@
     <hyperlink ref="C27" r:id="rId26"/>
     <hyperlink ref="C28" r:id="rId27"/>
     <hyperlink ref="C29" r:id="rId28"/>
-    <hyperlink ref="C30" r:id="rId29"/>
-    <hyperlink ref="C31" r:id="rId30"/>
-    <hyperlink ref="C32" r:id="rId31"/>
-    <hyperlink ref="C33" r:id="rId32"/>
-    <hyperlink ref="C34" r:id="rId33"/>
-    <hyperlink ref="C35" r:id="rId34"/>
-    <hyperlink ref="C36" r:id="rId35"/>
-    <hyperlink ref="C37" r:id="rId36"/>
   </hyperlinks>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Publish dashboard snapshot 2026-10-06 18:34
</commit_message>
<xml_diff>
--- a/assets/published-news.xlsx
+++ b/assets/published-news.xlsx
@@ -93,17 +93,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>www.nongup.net</t>
+          <t>www.yna.co.kr</t>
         </is>
       </c>
       <c r="C2" t="inlineStr" s="1">
         <is>
-          <t>거베라 소비 트렌드 바뀌었다…노동 부담 줄인 신품종 공개</t>
+          <t>한파특보 내려진 대관령</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>10월02일</t>
+          <t>10월06일</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -120,17 +120,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>news.bizwatch.co.kr</t>
+          <t>tjmbc.co.kr</t>
         </is>
       </c>
       <c r="C3" t="inlineStr" s="1">
         <is>
-          <t>네이버·컬리 '동맹 1년', 모두 웃었다 …다음 승부처는</t>
+          <t>[리포트]'돌풍에 쑥대밭' 비닐하우스..복구 중 죽은 작물은 보상 제외?</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>10월02일</t>
+          <t>10월06일</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -147,22 +147,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C4" t="inlineStr" s="1">
         <is>
-          <t>병해충 진단부터 영농기술 상담까지…‘AI 이삭이’ 2.0 출시</t>
+          <t>“밀식 재배에 유리한 호박 육종 빨라진다” 관련 분자표지 개발</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>10월02일</t>
+          <t>10월06일</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t/>
+          <t>한국농업기술진흥원</t>
         </is>
       </c>
     </row>
@@ -174,17 +174,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.kyongbuk.co.kr</t>
         </is>
       </c>
       <c r="C5" t="inlineStr" s="1">
         <is>
-          <t>가을에도 밭 갈아엎는다…‘양배추’ 농가에 무슨 일이?</t>
+          <t>예천군, 매실 퇴비·토착 미생물로 시설재배 토양 개선 나선다</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>10월02일</t>
+          <t>10월05일</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -201,17 +201,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>www.segye.com</t>
+          <t>www.joongboo.com</t>
         </is>
       </c>
       <c r="C6" t="inlineStr" s="1">
         <is>
-          <t>“종자 가치, 농업 시작 넘어 식량안보의 미래 결정”</t>
+          <t>절임 배추부터 양념·간편 키트까지…유통가 채비 나선 '김장 대전'</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>10월01일</t>
+          <t>10월05일</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -228,17 +228,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>www.obsnews.co.kr</t>
+          <t>biz.chosun.com</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="1">
         <is>
-          <t>도쿄 35일 연속 비 최장 기록…'기상병' 호소 증가</t>
+          <t>[뉴테크] 태양광과 농업, 두 마리 토끼 잡는다</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>10월01일</t>
+          <t>10월05일</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -255,17 +255,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>www.vegannews.co.kr</t>
+          <t>www.ohmynews.com</t>
         </is>
       </c>
       <c r="C8" t="inlineStr" s="1">
         <is>
-          <t>씨앗 봉투 발아율은 재배 성공률과 다르다</t>
+          <t>배추 묶어 놔야 속 찬다? 절대 안 됩니다</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>10월01일</t>
+          <t>10월04일</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -282,17 +282,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>www.ccdn.co.kr</t>
+          <t>www.vegannews.co.kr</t>
         </is>
       </c>
       <c r="C9" t="inlineStr" s="1">
         <is>
-          <t>충북농기원, 중소형 수박 신품종 보급 확대</t>
+          <t>토종 종자 보전, 수집부터 발아력 확인까지</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>10월01일</t>
+          <t>10월03일</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -309,17 +309,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>www.mbn.co.kr</t>
         </is>
       </c>
       <c r="C10" t="inlineStr" s="1">
         <is>
-          <t>본격적인 시설재배 시작, 바이러스병 예방해야</t>
+          <t>올겨울 깍두기 못 먹을라…배추 가격 떨어지는데 무는 '껑충'</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>10월01일</t>
+          <t>10월02일</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -336,17 +336,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>www.kyongbuk.co.kr</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C11" t="inlineStr" s="1">
         <is>
-          <t>성주 외국인 계절근로자 연말까지 970여 명 투입…농번기 인력난 지원</t>
+          <t>여름엔 폭염, 가을엔 생육 부진…고랭지 배추· 무 ‘이중고’</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>10월01일</t>
+          <t>10월02일</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -363,17 +363,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>www.gokorea.kr</t>
         </is>
       </c>
       <c r="C12" t="inlineStr" s="1">
         <is>
-          <t>영세성 갇힌 국내 종자 산업…"데이터 기반 신육종 지원 시급"</t>
+          <t>김장철 배추· 무 가격 작년보다 내렸다</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>10월01일</t>
+          <t>10월02일</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -390,17 +390,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>www.farmnmarket.com</t>
+          <t>www.hankyung.com</t>
         </is>
       </c>
       <c r="C13" t="inlineStr" s="1">
         <is>
-          <t>정읍시, 가을 배추· 무 병해충 초기 방제 당부</t>
+          <t>"밖에 나가기 싫다"…35일째 내린 비에 日경제까지 '직격탄' [도쿄나우]</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>10월01일</t>
+          <t>10월02일</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -417,17 +417,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>www.gasnews.com</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C14" t="inlineStr" s="1">
         <is>
-          <t>일본LP가스협회, 시설원예 난방연료로 LP가스 채택 확산</t>
+          <t>가을에도 밭 갈아엎는다…‘양배추’ 농가에 무슨 일이?</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>10월01일</t>
+          <t>10월02일</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -444,12 +444,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>www.kwnews.co.kr</t>
+          <t>www.segye.com</t>
         </is>
       </c>
       <c r="C15" t="inlineStr" s="1">
         <is>
-          <t>계절마다 농가 덮치는 이상기후⋯강원 농업 현장 ‘비상’</t>
+          <t>“종자 가치, 농업 시작 넘어 식량안보의 미래 결정”</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -471,17 +471,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>www.gnnews.co.kr</t>
+          <t>www.obsnews.co.kr</t>
         </is>
       </c>
       <c r="C16" t="inlineStr" s="1">
         <is>
-          <t>폭염에 빈 시설, 작은 수박 이 대안 될까</t>
+          <t>도쿄 35일 연속 비 최장 기록…'기상병' 호소 증가</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>09월30일</t>
+          <t>10월01일</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -498,17 +498,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>www.knnews.co.kr</t>
+          <t>www.vegannews.co.kr</t>
         </is>
       </c>
       <c r="C17" t="inlineStr" s="1">
         <is>
-          <t>경남농기원, 고온기 소과종 수박 수경재배 연구</t>
+          <t>씨앗 봉투 발아율은 재배 성공률과 다르다</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>09월30일</t>
+          <t>10월01일</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -525,17 +525,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>www.sisaweek.com</t>
+          <t>www.ccdn.co.kr</t>
         </is>
       </c>
       <c r="C18" t="inlineStr" s="1">
         <is>
-          <t>기후변화에 맞서는 '유전공학'… '식량난' 해법될까</t>
+          <t>충북농기원, 중소형 수박 신품종 보급 확대</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>09월30일</t>
+          <t>10월01일</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -552,22 +552,22 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C19" t="inlineStr" s="1">
         <is>
-          <t>바이러스, 매개충 차단과 불활성화로 이중 방어막 구축</t>
+          <t>본격적인 시설재배 시작, 바이러스병 예방해야</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>09월30일</t>
+          <t>10월01일</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>(주)경농</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -579,17 +579,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>www.m-i.kr</t>
+          <t>www.kyongbuk.co.kr</t>
         </is>
       </c>
       <c r="C20" t="inlineStr" s="1">
         <is>
-          <t>해남군, 시설과채류 줄기 유인 자동화…작업시간 47% 이상 단축</t>
+          <t>성주 외국인 계절근로자 연말까지 970여 명 투입…농번기 인력난 지원</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>09월30일</t>
+          <t>10월01일</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -606,22 +606,22 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>www.ilyoseoul.co.kr</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C21" t="inlineStr" s="1">
         <is>
-          <t>농협, 종자사업 통합 추진…NH농우바이오 중심 글로벌 경쟁력 강화</t>
+          <t>영세성 갇힌 국내 종자 산업…"데이터 기반 신육종 지원 시급"</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>09월30일</t>
+          <t>10월01일</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>농협종묘센터</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -633,17 +633,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>news.sbs.co.kr</t>
+          <t>www.farmnmarket.com</t>
         </is>
       </c>
       <c r="C22" t="inlineStr" s="1">
         <is>
-          <t>"벌써 김장철이네"…예년보다 빨라진 '예약 경쟁'</t>
+          <t>정읍시, 가을 배추· 무 병해충 초기 방제 당부</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>09월30일</t>
+          <t>10월01일</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -660,17 +660,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.gasnews.com</t>
         </is>
       </c>
       <c r="C23" t="inlineStr" s="1">
         <is>
-          <t>“내 손안의 인공지능(AI) 농사 전문가” 농촌진흥청, ‘AI 이삭이’ 2.0...</t>
+          <t>일본LP가스협회, 시설원예 난방연료로 LP가스 채택 확산</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>09월30일</t>
+          <t>10월01일</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -687,17 +687,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>www.youngnong.co.kr</t>
+          <t>www.kwnews.co.kr</t>
         </is>
       </c>
       <c r="C24" t="inlineStr" s="1">
         <is>
-          <t>NH농우바이오, 겨울 수박 ·참외 겨냥 10월 추천품종 4종 제안</t>
+          <t>계절마다 농가 덮치는 이상기후⋯강원 농업 현장 ‘비상’</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>09월30일</t>
+          <t>10월01일</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -714,12 +714,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>www.newsjeju.net</t>
+          <t>www.gnnews.co.kr</t>
         </is>
       </c>
       <c r="C25" t="inlineStr" s="1">
         <is>
-          <t>성산일출봉농협 청년부, 월동무 신품종 시험재배 실시</t>
+          <t>폭염에 빈 시설, 작은 수박 이 대안 될까</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -741,17 +741,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>www.youngnong.co.kr</t>
+          <t>www.knnews.co.kr</t>
         </is>
       </c>
       <c r="C26" t="inlineStr" s="1">
         <is>
-          <t>시설채소 바이러스병 비상…경농, 매개충 차단·바이러스 예방 '이중 방...</t>
+          <t>경남농기원, 고온기 소과종 수박 수경재배 연구</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>09월29일</t>
+          <t>09월30일</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -768,17 +768,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.sisaweek.com</t>
         </is>
       </c>
       <c r="C27" t="inlineStr" s="1">
         <is>
-          <t>한국원예학회 추계학술발표회 11월4~7일 제주서</t>
+          <t>기후변화에 맞서는 '유전공학'… '식량난' 해법될까</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>09월29일</t>
+          <t>09월30일</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -795,49 +795,22 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>www.newsfarm.co.kr</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C28" t="inlineStr" s="1">
         <is>
-          <t>팜한농, 가을철 안정 영농 위한 '맞춤형 3종' 주목</t>
+          <t>바이러스, 매개충 차단과 불활성화로 이중 방어막 구축</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>09월29일</t>
+          <t>09월30일</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>28</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>www.newsfarm.co.kr</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr" s="1">
-        <is>
-          <t>가을철 작물 위협 노균병·역병…체계적 관리 필요</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>09월29일</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t/>
+          <t>(주)경농</t>
         </is>
       </c>
     </row>
@@ -870,7 +843,6 @@
     <hyperlink ref="C26" r:id="rId25"/>
     <hyperlink ref="C27" r:id="rId26"/>
     <hyperlink ref="C28" r:id="rId27"/>
-    <hyperlink ref="C29" r:id="rId28"/>
   </hyperlinks>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Publish dashboard snapshot 2026-10-08 13:57
</commit_message>
<xml_diff>
--- a/assets/published-news.xlsx
+++ b/assets/published-news.xlsx
@@ -93,22 +93,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>www.yna.co.kr</t>
+          <t>www.wsobi.com</t>
         </is>
       </c>
       <c r="C2" t="inlineStr" s="1">
         <is>
-          <t>한파특보 내려진 대관령</t>
+          <t>건국대 '학생창업유망팀300+'서 대학 1위...신체장애인 위한 '스마트 치...</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>10월06일</t>
+          <t>10월08일</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t/>
+          <t>한국농업기술진흥원</t>
         </is>
       </c>
     </row>
@@ -120,22 +120,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>tjmbc.co.kr</t>
+          <t>news.kbs.co.kr</t>
         </is>
       </c>
       <c r="C3" t="inlineStr" s="1">
         <is>
-          <t>[리포트]'돌풍에 쑥대밭' 비닐하우스..복구 중 죽은 작물은 보상 제외?</t>
+          <t>농업 인 ‘관절을 지켜라’…‘무동력 입는 로봇’ 개발</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>10월06일</t>
+          <t>10월08일</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t/>
+          <t>한국농업기술진흥원</t>
         </is>
       </c>
     </row>
@@ -147,22 +147,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C4" t="inlineStr" s="1">
         <is>
-          <t>“밀식 재배에 유리한 호박 육종 빨라진다” 관련 분자표지 개발</t>
+          <t>고랭지 배추· 무 ‘생육 비상’…이상기후에 ‘고전’</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>10월06일</t>
+          <t>10월08일</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>한국농업기술진흥원</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -174,17 +174,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>www.kyongbuk.co.kr</t>
+          <t>www.ikpnews.net</t>
         </is>
       </c>
       <c r="C5" t="inlineStr" s="1">
         <is>
-          <t>예천군, 매실 퇴비·토착 미생물로 시설재배 토양 개선 나선다</t>
+          <t>내년 양파 공급 부족 우려…"재배면적 확대 필요"</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>10월05일</t>
+          <t>10월07일</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -201,17 +201,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>www.joongboo.com</t>
+          <t>www.gndomin.com</t>
         </is>
       </c>
       <c r="C6" t="inlineStr" s="1">
         <is>
-          <t>절임 배추부터 양념·간편 키트까지…유통가 채비 나선 '김장 대전'</t>
+          <t>남해군 "고품질 보물초 생산 위한 적정면적 파종"</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>10월05일</t>
+          <t>10월07일</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -228,17 +228,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>biz.chosun.com</t>
+          <t>www.yeongnam.com</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="1">
         <is>
-          <t>[뉴테크] 태양광과 농업, 두 마리 토끼 잡는다</t>
+          <t>“계절근로자 되려면 300만원”…농촌 파고든 해외 브로커</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>10월05일</t>
+          <t>10월07일</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -255,17 +255,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>www.ohmynews.com</t>
+          <t>www.hidomin.com</t>
         </is>
       </c>
       <c r="C8" t="inlineStr" s="1">
         <is>
-          <t>배추 묶어 놔야 속 찬다? 절대 안 됩니다</t>
+          <t>전국 종자 산업 공모 2곳 선정…경북도, 우량묘 생산 거점 확대</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>10월04일</t>
+          <t>10월07일</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -282,22 +282,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>www.vegannews.co.kr</t>
+          <t>www.wonyesanup.co.kr</t>
         </is>
       </c>
       <c r="C9" t="inlineStr" s="1">
         <is>
-          <t>토종 종자 보전, 수집부터 발아력 확인까지</t>
+          <t>농협 경제지주, 종자사업 통합</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>10월03일</t>
+          <t>10월07일</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t/>
+          <t>농협종묘센터</t>
         </is>
       </c>
     </row>
@@ -309,17 +309,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>www.mbn.co.kr</t>
+          <t>www.hankyung.com</t>
         </is>
       </c>
       <c r="C10" t="inlineStr" s="1">
         <is>
-          <t>올겨울 깍두기 못 먹을라…배추 가격 떨어지는데 무는 '껑충'</t>
+          <t>김용태 "농업 AI, 작황·기후 예측 대신…농가위법 단속에만 활용"</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>10월02일</t>
+          <t>10월07일</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -336,17 +336,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>view.asiae.co.kr</t>
         </is>
       </c>
       <c r="C11" t="inlineStr" s="1">
         <is>
-          <t>여름엔 폭염, 가을엔 생육 부진…고랭지 배추· 무 ‘이중고’</t>
+          <t>日 37일간 내린 비에 채솟값 인플레…"BOJ 정책에 영향 줄 수도"</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>10월02일</t>
+          <t>10월07일</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -363,17 +363,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>www.gokorea.kr</t>
+          <t>www.mk.co.kr</t>
         </is>
       </c>
       <c r="C12" t="inlineStr" s="1">
         <is>
-          <t>김장철 배추· 무 가격 작년보다 내렸다</t>
+          <t>농사일 돕는 로봇개 등장...20kg까지 거뜬히 운반</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>10월02일</t>
+          <t>10월07일</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -390,17 +390,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>www.hankyung.com</t>
+          <t>www.sedaily.com</t>
         </is>
       </c>
       <c r="C13" t="inlineStr" s="1">
         <is>
-          <t>"밖에 나가기 싫다"…35일째 내린 비에 日경제까지 '직격탄' [도쿄나우]</t>
+          <t>“중국산 아니면 괜찮겠지?” 베트남산 배추 검사했더니…농약 기준치...</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>10월02일</t>
+          <t>10월07일</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -422,12 +422,12 @@
       </c>
       <c r="C14" t="inlineStr" s="1">
         <is>
-          <t>가을에도 밭 갈아엎는다…‘양배추’ 농가에 무슨 일이?</t>
+          <t>기후변화 대응 겨울무 신품종 시범재배</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>10월02일</t>
+          <t>10월07일</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -444,22 +444,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>www.segye.com</t>
+          <t>news.kbs.co.kr</t>
         </is>
       </c>
       <c r="C15" t="inlineStr" s="1">
         <is>
-          <t>“종자 가치, 농업 시작 넘어 식량안보의 미래 결정”</t>
+          <t>새만금에 국내 최대 지능형 농기계 실증단지…“경쟁력·수출 제고 기대...</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>10월01일</t>
+          <t>10월06일</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t/>
+          <t>한국농업기술진흥원</t>
         </is>
       </c>
     </row>
@@ -471,17 +471,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>www.obsnews.co.kr</t>
+          <t>www.vegannews.co.kr</t>
         </is>
       </c>
       <c r="C16" t="inlineStr" s="1">
         <is>
-          <t>도쿄 35일 연속 비 최장 기록…'기상병' 호소 증가</t>
+          <t>농진청, 작물 생육 데이터 표준화 협의체 출범</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>10월01일</t>
+          <t>10월06일</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -498,22 +498,22 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>www.vegannews.co.kr</t>
+          <t>www.farmnmarket.com</t>
         </is>
       </c>
       <c r="C17" t="inlineStr" s="1">
         <is>
-          <t>씨앗 봉투 발아율은 재배 성공률과 다르다</t>
+          <t>호박 밀식재배 육종 빨라진다</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>10월01일</t>
+          <t>10월06일</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t/>
+          <t>한국농업기술진흥원</t>
         </is>
       </c>
     </row>
@@ -525,17 +525,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>www.ccdn.co.kr</t>
+          <t>www.farmnmarket.com</t>
         </is>
       </c>
       <c r="C18" t="inlineStr" s="1">
         <is>
-          <t>충북농기원, 중소형 수박 신품종 보급 확대</t>
+          <t>농업 위생관리, PAA 활용 주목</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>10월01일</t>
+          <t>10월06일</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -552,22 +552,22 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>www.newsfarm.co.kr</t>
         </is>
       </c>
       <c r="C19" t="inlineStr" s="1">
         <is>
-          <t>본격적인 시설재배 시작, 바이러스병 예방해야</t>
+          <t>경농, 시설채소 바이러스 '이중 방어' 나선다</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>10월01일</t>
+          <t>10월06일</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t/>
+          <t>(주)경농</t>
         </is>
       </c>
     </row>
@@ -579,17 +579,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>www.kyongbuk.co.kr</t>
+          <t>www.hortitimes.com</t>
         </is>
       </c>
       <c r="C20" t="inlineStr" s="1">
         <is>
-          <t>성주 외국인 계절근로자 연말까지 970여 명 투입…농번기 인력난 지원</t>
+          <t>10월 이달의 작물보호제</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>10월01일</t>
+          <t>10월06일</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -606,17 +606,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>www.yna.co.kr</t>
         </is>
       </c>
       <c r="C21" t="inlineStr" s="1">
         <is>
-          <t>영세성 갇힌 국내 종자 산업…"데이터 기반 신육종 지원 시급"</t>
+          <t>한파특보 내려진 대관령</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>10월01일</t>
+          <t>10월06일</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -633,17 +633,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>www.farmnmarket.com</t>
+          <t>tjmbc.co.kr</t>
         </is>
       </c>
       <c r="C22" t="inlineStr" s="1">
         <is>
-          <t>정읍시, 가을 배추· 무 병해충 초기 방제 당부</t>
+          <t>[리포트]'돌풍에 쑥대밭' 비닐하우스..복구 중 죽은 작물은 보상 제외?</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>10월01일</t>
+          <t>10월06일</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -660,17 +660,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>www.gasnews.com</t>
+          <t>www.kyongbuk.co.kr</t>
         </is>
       </c>
       <c r="C23" t="inlineStr" s="1">
         <is>
-          <t>일본LP가스협회, 시설원예 난방연료로 LP가스 채택 확산</t>
+          <t>예천군, 매실 퇴비·토착 미생물로 시설재배 토양 개선 나선다</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>10월01일</t>
+          <t>10월05일</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -687,17 +687,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>www.kwnews.co.kr</t>
+          <t>www.joongboo.com</t>
         </is>
       </c>
       <c r="C24" t="inlineStr" s="1">
         <is>
-          <t>계절마다 농가 덮치는 이상기후⋯강원 농업 현장 ‘비상’</t>
+          <t>절임 배추부터 양념·간편 키트까지…유통가 채비 나선 '김장 대전'</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>10월01일</t>
+          <t>10월05일</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -714,17 +714,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>www.gnnews.co.kr</t>
+          <t>biz.chosun.com</t>
         </is>
       </c>
       <c r="C25" t="inlineStr" s="1">
         <is>
-          <t>폭염에 빈 시설, 작은 수박 이 대안 될까</t>
+          <t>[뉴테크] 태양광과 농업, 두 마리 토끼 잡는다</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>09월30일</t>
+          <t>10월05일</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -741,17 +741,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>www.knnews.co.kr</t>
+          <t>www.ohmynews.com</t>
         </is>
       </c>
       <c r="C26" t="inlineStr" s="1">
         <is>
-          <t>경남농기원, 고온기 소과종 수박 수경재배 연구</t>
+          <t>배추 묶어 놔야 속 찬다? 절대 안 됩니다</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>09월30일</t>
+          <t>10월04일</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -768,17 +768,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>www.sisaweek.com</t>
+          <t>www.vegannews.co.kr</t>
         </is>
       </c>
       <c r="C27" t="inlineStr" s="1">
         <is>
-          <t>기후변화에 맞서는 '유전공학'… '식량난' 해법될까</t>
+          <t>토종 종자 보전, 수집부터 발아력 확인까지</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>09월30일</t>
+          <t>10월03일</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -795,22 +795,103 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.mbn.co.kr</t>
         </is>
       </c>
       <c r="C28" t="inlineStr" s="1">
         <is>
-          <t>바이러스, 매개충 차단과 불활성화로 이중 방어막 구축</t>
+          <t>올겨울 깍두기 못 먹을라…배추 가격 떨어지는데 무는 '껑충'</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>09월30일</t>
+          <t>10월02일</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>(주)경농</t>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>www.nongmin.com</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr" s="1">
+        <is>
+          <t>여름엔 폭염, 가을엔 생육 부진…고랭지 배추· 무 ‘이중고’</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>10월02일</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>www.gokorea.kr</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr" s="1">
+        <is>
+          <t>김장철 배추· 무 가격 작년보다 내렸다</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>10월02일</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>www.hankyung.com</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr" s="1">
+        <is>
+          <t>"밖에 나가기 싫다"…35일째 내린 비에 日경제까지 '직격탄' [도쿄나우]</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>10월02일</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t/>
         </is>
       </c>
     </row>
@@ -843,6 +924,9 @@
     <hyperlink ref="C26" r:id="rId25"/>
     <hyperlink ref="C27" r:id="rId26"/>
     <hyperlink ref="C28" r:id="rId27"/>
+    <hyperlink ref="C29" r:id="rId28"/>
+    <hyperlink ref="C30" r:id="rId29"/>
+    <hyperlink ref="C31" r:id="rId30"/>
   </hyperlinks>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Publish dashboard snapshot 2026-10-12 17:49
</commit_message>
<xml_diff>
--- a/assets/published-news.xlsx
+++ b/assets/published-news.xlsx
@@ -93,22 +93,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>www.wsobi.com</t>
+          <t>www.nongup.net</t>
         </is>
       </c>
       <c r="C2" t="inlineStr" s="1">
         <is>
-          <t>건국대 '학생창업유망팀300+'서 대학 1위...신체장애인 위한 '스마트 치...</t>
+          <t>무궁화 신품종 12종, 10월 9일부터 전국 판매 시작</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>10월08일</t>
+          <t>10월12일</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>한국농업기술진흥원</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -120,22 +120,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>news.kbs.co.kr</t>
+          <t>www.pinpointnews.co.kr</t>
         </is>
       </c>
       <c r="C3" t="inlineStr" s="1">
         <is>
-          <t>농업 인 ‘관절을 지켜라’…‘무동력 입는 로봇’ 개발</t>
+          <t>대동, 농업 관련 상장사 브랜드평판 1위…롯데정밀화학·남해화학 2·3위</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>10월08일</t>
+          <t>10월12일</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>한국농업기술진흥원</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -147,17 +147,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.g-enews.com</t>
         </is>
       </c>
       <c r="C4" t="inlineStr" s="1">
         <is>
-          <t>고랭지 배추· 무 ‘생육 비상’…이상기후에 ‘고전’</t>
+          <t>"전문가 경험 학습"… 中, 밀 우수 품종 선별 'AI 육종 로봇' 공개</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>10월08일</t>
+          <t>10월12일</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -174,17 +174,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>www.ikpnews.net</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C5" t="inlineStr" s="1">
         <is>
-          <t>내년 양파 공급 부족 우려…"재배면적 확대 필요"</t>
+          <t>농진청, 농생명 특화 거대언어모델 개발</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>10월07일</t>
+          <t>10월12일</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -201,17 +201,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>www.gndomin.com</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C6" t="inlineStr" s="1">
         <is>
-          <t>남해군 "고품질 보물초 생산 위한 적정면적 파종"</t>
+          <t>광활한 농지에 치솟는 생산비…호주농가 생존 전략은</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>10월07일</t>
+          <t>10월12일</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -228,17 +228,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>www.yeongnam.com</t>
+          <t>www.kado.net</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="1">
         <is>
-          <t>“계절근로자 되려면 300만원”…농촌 파고든 해외 브로커</t>
+          <t>공지천에 핀 '비밀의 정원' 13만 명 몰렸다</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>10월07일</t>
+          <t>10월12일</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -255,17 +255,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>www.hidomin.com</t>
+          <t>www.hankyung.com</t>
         </is>
       </c>
       <c r="C8" t="inlineStr" s="1">
         <is>
-          <t>전국 종자 산업 공모 2곳 선정…경북도, 우량묘 생산 거점 확대</t>
+          <t>'양배추가 양 상추 보다 비싸졌다'…뒤집힌 채소값 [프라이스&amp;]</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>10월07일</t>
+          <t>10월10일</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -282,22 +282,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>www.wonyesanup.co.kr</t>
+          <t>www.dongascience.com</t>
         </is>
       </c>
       <c r="C9" t="inlineStr" s="1">
         <is>
-          <t>농협 경제지주, 종자사업 통합</t>
+          <t>양상추 에서 동물성 단백질 생성…농사로 '고기' 재배할까</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>10월07일</t>
+          <t>10월10일</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>농협종묘센터</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -309,17 +309,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>www.hankyung.com</t>
+          <t>www.ppss.kr</t>
         </is>
       </c>
       <c r="C10" t="inlineStr" s="1">
         <is>
-          <t>김용태 "농업 AI, 작황·기후 예측 대신…농가위법 단속에만 활용"</t>
+          <t>국내 육성 신품종 꽃 한자리에…'2026 양재 플라워 페스타' 10월 개최</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>10월07일</t>
+          <t>10월09일</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -336,17 +336,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>view.asiae.co.kr</t>
+          <t>www.busan.com</t>
         </is>
       </c>
       <c r="C11" t="inlineStr" s="1">
         <is>
-          <t>日 37일간 내린 비에 채솟값 인플레…"BOJ 정책에 영향 줄 수도"</t>
+          <t>우수품종 경진대회, 배추 ‘청명가을’ 대통령상…기온 높아도 잘 자라</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>10월07일</t>
+          <t>10월08일</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -363,22 +363,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>www.mk.co.kr</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C12" t="inlineStr" s="1">
         <is>
-          <t>농사일 돕는 로봇개 등장...20kg까지 거뜬히 운반</t>
+          <t>동오그룹, 일본 J AGRI에서 선진 기술력 선보여</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>10월07일</t>
+          <t>10월08일</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t/>
+          <t>(주)경농</t>
         </is>
       </c>
     </row>
@@ -390,22 +390,22 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>www.sedaily.com</t>
+          <t>www.wsobi.com</t>
         </is>
       </c>
       <c r="C13" t="inlineStr" s="1">
         <is>
-          <t>“중국산 아니면 괜찮겠지?” 베트남산 배추 검사했더니…농약 기준치...</t>
+          <t>건국대 '학생창업유망팀300+'서 대학 1위...신체장애인 위한 '스마트 치...</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>10월07일</t>
+          <t>10월08일</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t/>
+          <t>한국농업기술진흥원</t>
         </is>
       </c>
     </row>
@@ -417,22 +417,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>news.kbs.co.kr</t>
         </is>
       </c>
       <c r="C14" t="inlineStr" s="1">
         <is>
-          <t>기후변화 대응 겨울무 신품종 시범재배</t>
+          <t>농업 인 ‘관절을 지켜라’…‘무동력 입는 로봇’ 개발</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>10월07일</t>
+          <t>10월08일</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t/>
+          <t>한국농업기술진흥원</t>
         </is>
       </c>
     </row>
@@ -444,22 +444,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>news.kbs.co.kr</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C15" t="inlineStr" s="1">
         <is>
-          <t>새만금에 국내 최대 지능형 농기계 실증단지…“경쟁력·수출 제고 기대...</t>
+          <t>고랭지 배추· 무 ‘생육 비상’…이상기후에 ‘고전’</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>10월06일</t>
+          <t>10월08일</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>한국농업기술진흥원</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -471,17 +471,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>www.vegannews.co.kr</t>
+          <t>www.ikpnews.net</t>
         </is>
       </c>
       <c r="C16" t="inlineStr" s="1">
         <is>
-          <t>농진청, 작물 생육 데이터 표준화 협의체 출범</t>
+          <t>내년 양파 공급 부족 우려…"재배면적 확대 필요"</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>10월06일</t>
+          <t>10월07일</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -498,22 +498,22 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>www.farmnmarket.com</t>
+          <t>www.gndomin.com</t>
         </is>
       </c>
       <c r="C17" t="inlineStr" s="1">
         <is>
-          <t>호박 밀식재배 육종 빨라진다</t>
+          <t>남해군 "고품질 보물초 생산 위한 적정면적 파종"</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>10월06일</t>
+          <t>10월07일</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>한국농업기술진흥원</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -525,17 +525,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>www.farmnmarket.com</t>
+          <t>www.yeongnam.com</t>
         </is>
       </c>
       <c r="C18" t="inlineStr" s="1">
         <is>
-          <t>농업 위생관리, PAA 활용 주목</t>
+          <t>“계절근로자 되려면 300만원”…농촌 파고든 해외 브로커</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>10월06일</t>
+          <t>10월07일</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -552,22 +552,22 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>www.newsfarm.co.kr</t>
+          <t>www.hidomin.com</t>
         </is>
       </c>
       <c r="C19" t="inlineStr" s="1">
         <is>
-          <t>경농, 시설채소 바이러스 '이중 방어' 나선다</t>
+          <t>전국 종자 산업 공모 2곳 선정…경북도, 우량묘 생산 거점 확대</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>10월06일</t>
+          <t>10월07일</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>(주)경농</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -579,22 +579,22 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>www.hortitimes.com</t>
+          <t>www.wonyesanup.co.kr</t>
         </is>
       </c>
       <c r="C20" t="inlineStr" s="1">
         <is>
-          <t>10월 이달의 작물보호제</t>
+          <t>농협 경제지주, 종자사업 통합</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>10월06일</t>
+          <t>10월07일</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t/>
+          <t>농협종묘센터</t>
         </is>
       </c>
     </row>
@@ -606,17 +606,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>www.yna.co.kr</t>
+          <t>www.hankyung.com</t>
         </is>
       </c>
       <c r="C21" t="inlineStr" s="1">
         <is>
-          <t>한파특보 내려진 대관령</t>
+          <t>김용태 "농업 AI, 작황·기후 예측 대신…농가위법 단속에만 활용"</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>10월06일</t>
+          <t>10월07일</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -633,17 +633,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>tjmbc.co.kr</t>
+          <t>view.asiae.co.kr</t>
         </is>
       </c>
       <c r="C22" t="inlineStr" s="1">
         <is>
-          <t>[리포트]'돌풍에 쑥대밭' 비닐하우스..복구 중 죽은 작물은 보상 제외?</t>
+          <t>日 37일간 내린 비에 채솟값 인플레…"BOJ 정책에 영향 줄 수도"</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>10월06일</t>
+          <t>10월07일</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -660,17 +660,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>www.kyongbuk.co.kr</t>
+          <t>www.mk.co.kr</t>
         </is>
       </c>
       <c r="C23" t="inlineStr" s="1">
         <is>
-          <t>예천군, 매실 퇴비·토착 미생물로 시설재배 토양 개선 나선다</t>
+          <t>농사일 돕는 로봇개 등장...20kg까지 거뜬히 운반</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>10월05일</t>
+          <t>10월07일</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -687,17 +687,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>www.joongboo.com</t>
+          <t>www.sedaily.com</t>
         </is>
       </c>
       <c r="C24" t="inlineStr" s="1">
         <is>
-          <t>절임 배추부터 양념·간편 키트까지…유통가 채비 나선 '김장 대전'</t>
+          <t>“중국산 아니면 괜찮겠지?” 베트남산 배추 검사했더니…농약 기준치...</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>10월05일</t>
+          <t>10월07일</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -714,17 +714,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>biz.chosun.com</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C25" t="inlineStr" s="1">
         <is>
-          <t>[뉴테크] 태양광과 농업, 두 마리 토끼 잡는다</t>
+          <t>기후변화 대응 겨울무 신품종 시범재배</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>10월05일</t>
+          <t>10월07일</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -741,22 +741,22 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>www.ohmynews.com</t>
+          <t>news.kbs.co.kr</t>
         </is>
       </c>
       <c r="C26" t="inlineStr" s="1">
         <is>
-          <t>배추 묶어 놔야 속 찬다? 절대 안 됩니다</t>
+          <t>새만금에 국내 최대 지능형 농기계 실증단지…“경쟁력·수출 제고 기대...</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>10월04일</t>
+          <t>10월06일</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t/>
+          <t>한국농업기술진흥원</t>
         </is>
       </c>
     </row>
@@ -773,12 +773,12 @@
       </c>
       <c r="C27" t="inlineStr" s="1">
         <is>
-          <t>토종 종자 보전, 수집부터 발아력 확인까지</t>
+          <t>농진청, 작물 생육 데이터 표준화 협의체 출범</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>10월03일</t>
+          <t>10월06일</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -795,17 +795,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>www.mbn.co.kr</t>
+          <t>www.farmnmarket.com</t>
         </is>
       </c>
       <c r="C28" t="inlineStr" s="1">
         <is>
-          <t>올겨울 깍두기 못 먹을라…배추 가격 떨어지는데 무는 '껑충'</t>
+          <t>호박 밀식재배 육종 빨라진다</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>10월02일</t>
+          <t>10월06일</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -822,17 +822,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.farmnmarket.com</t>
         </is>
       </c>
       <c r="C29" t="inlineStr" s="1">
         <is>
-          <t>여름엔 폭염, 가을엔 생육 부진…고랭지 배추· 무 ‘이중고’</t>
+          <t>농업 위생관리, PAA 활용 주목</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>10월02일</t>
+          <t>10월06일</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -849,22 +849,22 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>www.gokorea.kr</t>
+          <t>www.newsfarm.co.kr</t>
         </is>
       </c>
       <c r="C30" t="inlineStr" s="1">
         <is>
-          <t>김장철 배추· 무 가격 작년보다 내렸다</t>
+          <t>경농, 시설채소 바이러스 '이중 방어' 나선다</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>10월02일</t>
+          <t>10월06일</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t/>
+          <t>(주)경농</t>
         </is>
       </c>
     </row>
@@ -876,20 +876,101 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>www.hankyung.com</t>
+          <t>www.hortitimes.com</t>
         </is>
       </c>
       <c r="C31" t="inlineStr" s="1">
         <is>
-          <t>"밖에 나가기 싫다"…35일째 내린 비에 日경제까지 '직격탄' [도쿄나우]</t>
+          <t>10월 이달의 작물보호제</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
+          <t>10월06일</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>www.ohmynews.com</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr" s="1">
+        <is>
+          <t>배추 묶어 놔야 속 찬다? 절대 안 됩니다</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>10월04일</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>www.vegannews.co.kr</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr" s="1">
+        <is>
+          <t>토종 종자 보전, 수집부터 발아력 확인까지</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>10월03일</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>www.mbn.co.kr</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr" s="1">
+        <is>
+          <t>올겨울 깍두기 못 먹을라…배추 가격 떨어지는데 무는 '껑충'</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
           <t>10월02일</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr">
+      <c r="E34" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -927,6 +1008,9 @@
     <hyperlink ref="C29" r:id="rId28"/>
     <hyperlink ref="C30" r:id="rId29"/>
     <hyperlink ref="C31" r:id="rId30"/>
+    <hyperlink ref="C32" r:id="rId31"/>
+    <hyperlink ref="C33" r:id="rId32"/>
+    <hyperlink ref="C34" r:id="rId33"/>
   </hyperlinks>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Publish dashboard snapshot 2026-10-13 15:55
</commit_message>
<xml_diff>
--- a/assets/published-news.xlsx
+++ b/assets/published-news.xlsx
@@ -93,22 +93,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>www.nongup.net</t>
+          <t>www.farmnmarket.com</t>
         </is>
       </c>
       <c r="C2" t="inlineStr" s="1">
         <is>
-          <t>무궁화 신품종 12종, 10월 9일부터 전국 판매 시작</t>
+          <t>농업기술, 도시의 일상으로 확장</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>10월12일</t>
+          <t>10월13일</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t/>
+          <t>(주)팜한농</t>
         </is>
       </c>
     </row>
@@ -120,12 +120,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>www.pinpointnews.co.kr</t>
+          <t>www.cstimes.com</t>
         </is>
       </c>
       <c r="C3" t="inlineStr" s="1">
         <is>
-          <t>대동, 농업 관련 상장사 브랜드평판 1위…롯데정밀화학·남해화학 2·3위</t>
+          <t>농수산식품유통공사(aT), 16일 '제8회 양재 플라워 페스타' 개막</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -147,12 +147,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>www.g-enews.com</t>
+          <t>www.hansbiz.co.kr</t>
         </is>
       </c>
       <c r="C4" t="inlineStr" s="1">
         <is>
-          <t>"전문가 경험 학습"… 中, 밀 우수 품종 선별 'AI 육종 로봇' 공개</t>
+          <t>아시아종묘, 배추 신 품종 5종 출원</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -174,12 +174,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>www.aflnews.co.kr</t>
+          <t>www.abcn.kr</t>
         </is>
       </c>
       <c r="C5" t="inlineStr" s="1">
         <is>
-          <t>농진청, 농생명 특화 거대언어모델 개발</t>
+          <t>내년 시금치 값 더 떨어지나...남해 보물초 재배면적 20% 급증 전망</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -201,12 +201,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.nongup.net</t>
         </is>
       </c>
       <c r="C6" t="inlineStr" s="1">
         <is>
-          <t>광활한 농지에 치솟는 생산비…호주농가 생존 전략은</t>
+          <t>무궁화 신품종 12종, 10월 9일부터 전국 판매 시작</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -228,12 +228,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>www.kado.net</t>
+          <t>www.pinpointnews.co.kr</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="1">
         <is>
-          <t>공지천에 핀 '비밀의 정원' 13만 명 몰렸다</t>
+          <t>대동, 농업 관련 상장사 브랜드평판 1위…롯데정밀화학·남해화학 2·3위</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -255,17 +255,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>www.hankyung.com</t>
+          <t>www.g-enews.com</t>
         </is>
       </c>
       <c r="C8" t="inlineStr" s="1">
         <is>
-          <t>'양배추가 양 상추 보다 비싸졌다'…뒤집힌 채소값 [프라이스&amp;]</t>
+          <t>"전문가 경험 학습"… 中, 밀 우수 품종 선별 'AI 육종 로봇' 공개</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>10월10일</t>
+          <t>10월12일</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -282,17 +282,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>www.dongascience.com</t>
+          <t>www.aflnews.co.kr</t>
         </is>
       </c>
       <c r="C9" t="inlineStr" s="1">
         <is>
-          <t>양상추 에서 동물성 단백질 생성…농사로 '고기' 재배할까</t>
+          <t>농진청, 농생명 특화 거대언어모델 개발</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>10월10일</t>
+          <t>10월12일</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -309,17 +309,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>www.ppss.kr</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C10" t="inlineStr" s="1">
         <is>
-          <t>국내 육성 신품종 꽃 한자리에…'2026 양재 플라워 페스타' 10월 개최</t>
+          <t>광활한 농지에 치솟는 생산비…호주농가 생존 전략은</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>10월09일</t>
+          <t>10월12일</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -336,17 +336,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>www.busan.com</t>
+          <t>www.kado.net</t>
         </is>
       </c>
       <c r="C11" t="inlineStr" s="1">
         <is>
-          <t>우수품종 경진대회, 배추 ‘청명가을’ 대통령상…기온 높아도 잘 자라</t>
+          <t>공지천에 핀 '비밀의 정원' 13만 명 몰렸다</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>10월08일</t>
+          <t>10월12일</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -363,22 +363,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>www.newsam.co.kr</t>
+          <t>www.hankyung.com</t>
         </is>
       </c>
       <c r="C12" t="inlineStr" s="1">
         <is>
-          <t>동오그룹, 일본 J AGRI에서 선진 기술력 선보여</t>
+          <t>'양배추가 양 상추 보다 비싸졌다'…뒤집힌 채소값 [프라이스&amp;]</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>10월08일</t>
+          <t>10월10일</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>(주)경농</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -390,22 +390,22 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>www.wsobi.com</t>
+          <t>www.dongascience.com</t>
         </is>
       </c>
       <c r="C13" t="inlineStr" s="1">
         <is>
-          <t>건국대 '학생창업유망팀300+'서 대학 1위...신체장애인 위한 '스마트 치...</t>
+          <t>양상추 에서 동물성 단백질 생성…농사로 '고기' 재배할까</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>10월08일</t>
+          <t>10월10일</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>한국농업기술진흥원</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -417,22 +417,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>news.kbs.co.kr</t>
+          <t>www.ppss.kr</t>
         </is>
       </c>
       <c r="C14" t="inlineStr" s="1">
         <is>
-          <t>농업 인 ‘관절을 지켜라’…‘무동력 입는 로봇’ 개발</t>
+          <t>국내 육성 신품종 꽃 한자리에…'2026 양재 플라워 페스타' 10월 개최</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>10월08일</t>
+          <t>10월09일</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>한국농업기술진흥원</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -444,12 +444,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.busan.com</t>
         </is>
       </c>
       <c r="C15" t="inlineStr" s="1">
         <is>
-          <t>고랭지 배추· 무 ‘생육 비상’…이상기후에 ‘고전’</t>
+          <t>우수품종 경진대회, 배추 ‘청명가을’ 대통령상…기온 높아도 잘 자라</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -471,22 +471,22 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>www.ikpnews.net</t>
+          <t>www.newsam.co.kr</t>
         </is>
       </c>
       <c r="C16" t="inlineStr" s="1">
         <is>
-          <t>내년 양파 공급 부족 우려…"재배면적 확대 필요"</t>
+          <t>동오그룹, 일본 J AGRI에서 선진 기술력 선보여</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>10월07일</t>
+          <t>10월08일</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t/>
+          <t>(주)경농</t>
         </is>
       </c>
     </row>
@@ -498,17 +498,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>www.gndomin.com</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C17" t="inlineStr" s="1">
         <is>
-          <t>남해군 "고품질 보물초 생산 위한 적정면적 파종"</t>
+          <t>고랭지 배추· 무 ‘생육 비상’…이상기후에 ‘고전’</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>10월07일</t>
+          <t>10월08일</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -525,12 +525,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>www.yeongnam.com</t>
+          <t>www.ikpnews.net</t>
         </is>
       </c>
       <c r="C18" t="inlineStr" s="1">
         <is>
-          <t>“계절근로자 되려면 300만원”…농촌 파고든 해외 브로커</t>
+          <t>내년 양파 공급 부족 우려…"재배면적 확대 필요"</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -552,12 +552,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>www.hidomin.com</t>
+          <t>www.gndomin.com</t>
         </is>
       </c>
       <c r="C19" t="inlineStr" s="1">
         <is>
-          <t>전국 종자 산업 공모 2곳 선정…경북도, 우량묘 생산 거점 확대</t>
+          <t>남해군 "고품질 보물초 생산 위한 적정면적 파종"</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -579,12 +579,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>www.wonyesanup.co.kr</t>
+          <t>www.yeongnam.com</t>
         </is>
       </c>
       <c r="C20" t="inlineStr" s="1">
         <is>
-          <t>농협 경제지주, 종자사업 통합</t>
+          <t>“계절근로자 되려면 300만원”…농촌 파고든 해외 브로커</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -594,7 +594,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>농협종묘센터</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -606,12 +606,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>www.hankyung.com</t>
+          <t>www.hidomin.com</t>
         </is>
       </c>
       <c r="C21" t="inlineStr" s="1">
         <is>
-          <t>김용태 "농업 AI, 작황·기후 예측 대신…농가위법 단속에만 활용"</t>
+          <t>전국 종자 산업 공모 2곳 선정…경북도, 우량묘 생산 거점 확대</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -633,12 +633,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>view.asiae.co.kr</t>
+          <t>www.wonyesanup.co.kr</t>
         </is>
       </c>
       <c r="C22" t="inlineStr" s="1">
         <is>
-          <t>日 37일간 내린 비에 채솟값 인플레…"BOJ 정책에 영향 줄 수도"</t>
+          <t>농협 경제지주, 종자사업 통합</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -648,7 +648,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t/>
+          <t>농협종묘센터</t>
         </is>
       </c>
     </row>
@@ -660,12 +660,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>www.mk.co.kr</t>
+          <t>www.hankyung.com</t>
         </is>
       </c>
       <c r="C23" t="inlineStr" s="1">
         <is>
-          <t>농사일 돕는 로봇개 등장...20kg까지 거뜬히 운반</t>
+          <t>김용태 "농업 AI, 작황·기후 예측 대신…농가위법 단속에만 활용"</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -687,12 +687,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>www.sedaily.com</t>
+          <t>view.asiae.co.kr</t>
         </is>
       </c>
       <c r="C24" t="inlineStr" s="1">
         <is>
-          <t>“중국산 아니면 괜찮겠지?” 베트남산 배추 검사했더니…농약 기준치...</t>
+          <t>日 37일간 내린 비에 채솟값 인플레…"BOJ 정책에 영향 줄 수도"</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -714,12 +714,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>www.nongmin.com</t>
+          <t>www.mk.co.kr</t>
         </is>
       </c>
       <c r="C25" t="inlineStr" s="1">
         <is>
-          <t>기후변화 대응 겨울무 신품종 시범재배</t>
+          <t>농사일 돕는 로봇개 등장...20kg까지 거뜬히 운반</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -741,22 +741,22 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>news.kbs.co.kr</t>
+          <t>www.sedaily.com</t>
         </is>
       </c>
       <c r="C26" t="inlineStr" s="1">
         <is>
-          <t>새만금에 국내 최대 지능형 농기계 실증단지…“경쟁력·수출 제고 기대...</t>
+          <t>“중국산 아니면 괜찮겠지?” 베트남산 배추 검사했더니…농약 기준치...</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>10월06일</t>
+          <t>10월07일</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>한국농업기술진흥원</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -768,17 +768,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>www.vegannews.co.kr</t>
+          <t>www.nongmin.com</t>
         </is>
       </c>
       <c r="C27" t="inlineStr" s="1">
         <is>
-          <t>농진청, 작물 생육 데이터 표준화 협의체 출범</t>
+          <t>기후변화 대응 겨울무 신품종 시범재배</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>10월06일</t>
+          <t>10월07일</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -795,12 +795,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>www.farmnmarket.com</t>
+          <t>news.kbs.co.kr</t>
         </is>
       </c>
       <c r="C28" t="inlineStr" s="1">
         <is>
-          <t>호박 밀식재배 육종 빨라진다</t>
+          <t>새만금에 국내 최대 지능형 농기계 실증단지…“경쟁력·수출 제고 기대...</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -810,7 +810,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t/>
+          <t>한국농업기술진흥원</t>
         </is>
       </c>
     </row>
@@ -822,12 +822,12 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>www.farmnmarket.com</t>
+          <t>www.vegannews.co.kr</t>
         </is>
       </c>
       <c r="C29" t="inlineStr" s="1">
         <is>
-          <t>농업 위생관리, PAA 활용 주목</t>
+          <t>농진청, 작물 생육 데이터 표준화 협의체 출범</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -849,12 +849,12 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>www.newsfarm.co.kr</t>
+          <t>www.farmnmarket.com</t>
         </is>
       </c>
       <c r="C30" t="inlineStr" s="1">
         <is>
-          <t>경농, 시설채소 바이러스 '이중 방어' 나선다</t>
+          <t>호박 밀식재배 육종 빨라진다</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -864,7 +864,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>(주)경농</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -876,12 +876,12 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>www.hortitimes.com</t>
+          <t>www.farmnmarket.com</t>
         </is>
       </c>
       <c r="C31" t="inlineStr" s="1">
         <is>
-          <t>10월 이달의 작물보호제</t>
+          <t>농업 위생관리, PAA 활용 주목</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -903,22 +903,22 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>www.ohmynews.com</t>
+          <t>www.newsfarm.co.kr</t>
         </is>
       </c>
       <c r="C32" t="inlineStr" s="1">
         <is>
-          <t>배추 묶어 놔야 속 찬다? 절대 안 됩니다</t>
+          <t>경농, 시설채소 바이러스 '이중 방어' 나선다</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>10월04일</t>
+          <t>10월06일</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t/>
+          <t>(주)경농</t>
         </is>
       </c>
     </row>
@@ -930,47 +930,20 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>www.vegannews.co.kr</t>
+          <t>www.hortitimes.com</t>
         </is>
       </c>
       <c r="C33" t="inlineStr" s="1">
         <is>
-          <t>토종 종자 보전, 수집부터 발아력 확인까지</t>
+          <t>10월 이달의 작물보호제</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>10월03일</t>
+          <t>10월06일</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>33</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>www.mbn.co.kr</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr" s="1">
-        <is>
-          <t>올겨울 깍두기 못 먹을라…배추 가격 떨어지는데 무는 '껑충'</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>10월02일</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -1010,7 +983,6 @@
     <hyperlink ref="C31" r:id="rId30"/>
     <hyperlink ref="C32" r:id="rId31"/>
     <hyperlink ref="C33" r:id="rId32"/>
-    <hyperlink ref="C34" r:id="rId33"/>
   </hyperlinks>
 </worksheet>
 </file>
</xml_diff>